<commit_message>
Fix scroll reset on periodic re-render; reduce Raid Epic weapon rate at Lv8-10
- Fix Inventory/Collection/equip screens snapping scroll to top every time a
  background tick (resting regen, stamina regen) triggers a full re-render.
  render() now saves and restores scrollTop of every overflow-y:auto container
  across the innerHTML replacement.
- Reduce Raid weapon Epic drop rate at Level 8-10 (23/32/45% -> 20/25/30%),
  redistributing the difference into Rare (42/43/40% -> 45/50/55%); Normal
  rate unchanged. Sync SYMBEAST_Evolve_Forms.xlsx Raid Rewards sheet to match.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SYMBEAST_Evolve_Forms.xlsx
+++ b/SYMBEAST_Evolve_Forms.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\skyit\Desktop\Symbeast-main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65711DEB-68B4-4330-A764-22A77FC06920}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A144408-308F-45E6-BBF4-CD63EAA0DFF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2607" uniqueCount="1660">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2601" uniqueCount="1656">
   <si>
     <t>SYMBEAST — Evolved Forms (Stage 1, 10 forms)</t>
   </si>
@@ -4065,18 +4065,6 @@
   </si>
   <si>
     <t>39%</t>
-  </si>
-  <si>
-    <t>42%</t>
-  </si>
-  <si>
-    <t>23%</t>
-  </si>
-  <si>
-    <t>43%</t>
-  </si>
-  <si>
-    <t>32%</t>
   </si>
   <si>
     <t>Weapon การันตี 1 ชิ้นทุกครั้งที่ชนะ Wave 3 (บอสพิเศษ) — เกรดสุ่มตามตาราง</t>
@@ -5048,9 +5036,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -8055,11 +8044,11 @@
       <c r="B62" t="s">
         <v>918</v>
       </c>
-      <c r="C62" t="s">
-        <v>1344</v>
-      </c>
-      <c r="D62" t="s">
-        <v>1345</v>
+      <c r="C62" s="2">
+        <v>0.45</v>
+      </c>
+      <c r="D62" s="2">
+        <v>0.2</v>
       </c>
     </row>
     <row r="63" spans="1:13" x14ac:dyDescent="0.3">
@@ -8069,11 +8058,11 @@
       <c r="B63" t="s">
         <v>905</v>
       </c>
-      <c r="C63" t="s">
-        <v>1346</v>
-      </c>
-      <c r="D63" t="s">
-        <v>1347</v>
+      <c r="C63" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="D63" s="2">
+        <v>0.25</v>
       </c>
     </row>
     <row r="64" spans="1:13" x14ac:dyDescent="0.3">
@@ -8083,21 +8072,21 @@
       <c r="B64" t="s">
         <v>976</v>
       </c>
-      <c r="C64" t="s">
-        <v>1012</v>
-      </c>
-      <c r="D64" t="s">
-        <v>1342</v>
+      <c r="C64" s="2">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="D64" s="2">
+        <v>0.3</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>1348</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>1349</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.3">
@@ -8105,19 +8094,19 @@
         <v>1331</v>
       </c>
       <c r="B69" t="s">
+        <v>1346</v>
+      </c>
+      <c r="C69" t="s">
+        <v>1347</v>
+      </c>
+      <c r="D69" t="s">
+        <v>1348</v>
+      </c>
+      <c r="E69" t="s">
+        <v>1349</v>
+      </c>
+      <c r="F69" t="s">
         <v>1350</v>
-      </c>
-      <c r="C69" t="s">
-        <v>1351</v>
-      </c>
-      <c r="D69" t="s">
-        <v>1352</v>
-      </c>
-      <c r="E69" t="s">
-        <v>1353</v>
-      </c>
-      <c r="F69" t="s">
-        <v>1354</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.3">
@@ -8145,7 +8134,7 @@
         <v>985</v>
       </c>
       <c r="B71" t="s">
-        <v>1355</v>
+        <v>1351</v>
       </c>
       <c r="C71" t="s">
         <v>910</v>
@@ -8185,7 +8174,7 @@
         <v>979</v>
       </c>
       <c r="B73" t="s">
-        <v>1356</v>
+        <v>1352</v>
       </c>
       <c r="C73" t="s">
         <v>910</v>
@@ -8194,7 +8183,7 @@
         <v>910</v>
       </c>
       <c r="E73" t="s">
-        <v>1357</v>
+        <v>1353</v>
       </c>
       <c r="F73" t="s">
         <v>913</v>
@@ -8205,7 +8194,7 @@
         <v>978</v>
       </c>
       <c r="B74" t="s">
-        <v>1358</v>
+        <v>1354</v>
       </c>
       <c r="C74" t="s">
         <v>980</v>
@@ -8234,10 +8223,10 @@
         <v>910</v>
       </c>
       <c r="E75" t="s">
-        <v>1359</v>
+        <v>1355</v>
       </c>
       <c r="F75" t="s">
-        <v>1360</v>
+        <v>1356</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.3">
@@ -8245,7 +8234,7 @@
         <v>1309</v>
       </c>
       <c r="B76" t="s">
-        <v>1361</v>
+        <v>1357</v>
       </c>
       <c r="C76" t="s">
         <v>984</v>
@@ -8265,7 +8254,7 @@
         <v>983</v>
       </c>
       <c r="B77" t="s">
-        <v>1362</v>
+        <v>1358</v>
       </c>
       <c r="C77" t="s">
         <v>908</v>
@@ -8274,10 +8263,10 @@
         <v>986</v>
       </c>
       <c r="E77" t="s">
-        <v>1363</v>
+        <v>1359</v>
       </c>
       <c r="F77" t="s">
-        <v>1355</v>
+        <v>1351</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.3">
@@ -8285,7 +8274,7 @@
         <v>1312</v>
       </c>
       <c r="B78" t="s">
-        <v>1364</v>
+        <v>1360</v>
       </c>
       <c r="C78" t="s">
         <v>1041</v>
@@ -8294,7 +8283,7 @@
         <v>980</v>
       </c>
       <c r="E78" t="s">
-        <v>1365</v>
+        <v>1361</v>
       </c>
       <c r="F78" t="s">
         <v>976</v>
@@ -8305,7 +8294,7 @@
         <v>977</v>
       </c>
       <c r="B79" t="s">
-        <v>1366</v>
+        <v>1362</v>
       </c>
       <c r="C79" t="s">
         <v>1019</v>
@@ -8322,18 +8311,18 @@
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
-        <v>1367</v>
+        <v>1363</v>
       </c>
     </row>
     <row r="82" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
-        <v>1368</v>
+        <v>1364</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:M82" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:M61 A65:M82 A62:B62 E62:M62 A63:B63 E63:M63 A64:B64 E64:M64" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -8345,17 +8334,17 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>1369</v>
+        <v>1365</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>1370</v>
+        <v>1366</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>1371</v>
+        <v>1367</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
@@ -8371,7 +8360,7 @@
         <v>1263</v>
       </c>
       <c r="B6" t="s">
-        <v>1372</v>
+        <v>1368</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
@@ -8379,23 +8368,23 @@
         <v>1265</v>
       </c>
       <c r="B7" t="s">
-        <v>1373</v>
+        <v>1369</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>1374</v>
+        <v>1370</v>
       </c>
       <c r="B8" t="s">
-        <v>1375</v>
+        <v>1371</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>1376</v>
+        <v>1372</v>
       </c>
       <c r="B9" t="s">
-        <v>1377</v>
+        <v>1373</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
@@ -8403,7 +8392,7 @@
         <v>1277</v>
       </c>
       <c r="B10" t="s">
-        <v>1378</v>
+        <v>1374</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
@@ -8411,157 +8400,157 @@
         <v>1279</v>
       </c>
       <c r="B11" t="s">
-        <v>1379</v>
+        <v>1375</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>1380</v>
+        <v>1376</v>
       </c>
       <c r="B12" t="s">
-        <v>1381</v>
+        <v>1377</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>1382</v>
+        <v>1378</v>
       </c>
       <c r="B13" t="s">
-        <v>1383</v>
+        <v>1379</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>1384</v>
+        <v>1380</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>1385</v>
+        <v>1381</v>
       </c>
       <c r="B16" t="s">
-        <v>1386</v>
+        <v>1382</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>1387</v>
+        <v>1383</v>
       </c>
       <c r="B17" t="s">
-        <v>1388</v>
+        <v>1384</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>1389</v>
+        <v>1385</v>
       </c>
       <c r="B18" t="s">
-        <v>1390</v>
+        <v>1386</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>1391</v>
+        <v>1387</v>
       </c>
       <c r="B19" t="s">
-        <v>1392</v>
+        <v>1388</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>1393</v>
+        <v>1389</v>
       </c>
       <c r="B20" t="s">
-        <v>1394</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>1395</v>
+        <v>1391</v>
       </c>
       <c r="B22" t="s">
-        <v>1396</v>
+        <v>1392</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>1397</v>
+        <v>1393</v>
       </c>
       <c r="B23" t="s">
-        <v>1398</v>
+        <v>1394</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>1399</v>
+        <v>1395</v>
       </c>
       <c r="B24" t="s">
-        <v>1400</v>
+        <v>1396</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>1401</v>
+        <v>1397</v>
       </c>
       <c r="B25" t="s">
-        <v>1402</v>
+        <v>1398</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>1403</v>
+        <v>1399</v>
       </c>
       <c r="B26" t="s">
-        <v>1404</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>1405</v>
+        <v>1401</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>1406</v>
+        <v>1402</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>1395</v>
+        <v>1391</v>
       </c>
       <c r="B31" t="s">
-        <v>1407</v>
+        <v>1403</v>
       </c>
       <c r="C31" t="s">
-        <v>1408</v>
+        <v>1404</v>
       </c>
       <c r="D31" t="s">
-        <v>1409</v>
+        <v>1405</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>1410</v>
+        <v>1406</v>
       </c>
       <c r="B32" t="s">
-        <v>1411</v>
+        <v>1407</v>
       </c>
       <c r="C32" t="s">
-        <v>1411</v>
+        <v>1407</v>
       </c>
       <c r="D32" t="s">
-        <v>1412</v>
+        <v>1408</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>1413</v>
+        <v>1409</v>
       </c>
       <c r="B33" t="s">
-        <v>1414</v>
+        <v>1410</v>
       </c>
       <c r="C33" t="s">
-        <v>1411</v>
+        <v>1407</v>
       </c>
       <c r="D33" t="s">
         <v>906</v>
@@ -8569,77 +8558,77 @@
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>1415</v>
+        <v>1411</v>
       </c>
       <c r="B34" t="s">
-        <v>1414</v>
+        <v>1410</v>
       </c>
       <c r="C34" t="s">
-        <v>1414</v>
+        <v>1410</v>
       </c>
       <c r="D34" t="s">
-        <v>1416</v>
+        <v>1412</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>1417</v>
+        <v>1413</v>
       </c>
       <c r="B35" t="s">
-        <v>1411</v>
+        <v>1407</v>
       </c>
       <c r="C35" t="s">
-        <v>1418</v>
+        <v>1414</v>
       </c>
       <c r="D35" t="s">
-        <v>1419</v>
+        <v>1415</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>1420</v>
+        <v>1416</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>1421</v>
+        <v>1417</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>1422</v>
+        <v>1418</v>
       </c>
       <c r="B40" t="s">
-        <v>1423</v>
+        <v>1419</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>1424</v>
+        <v>1420</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>1395</v>
+        <v>1391</v>
       </c>
       <c r="B43" t="s">
-        <v>1425</v>
+        <v>1421</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>1426</v>
+        <v>1422</v>
       </c>
       <c r="B44" t="s">
-        <v>1427</v>
+        <v>1423</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>1428</v>
+        <v>1424</v>
       </c>
       <c r="B45" t="s">
-        <v>1429</v>
+        <v>1425</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.3">
@@ -8647,17 +8636,17 @@
         <v>1314</v>
       </c>
       <c r="B46" t="s">
-        <v>1430</v>
+        <v>1426</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>1431</v>
+        <v>1427</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>1432</v>
+        <v>1428</v>
       </c>
       <c r="B50" t="s">
         <v>944</v>
@@ -8668,15 +8657,15 @@
         <v>977</v>
       </c>
       <c r="B51" t="s">
-        <v>1433</v>
+        <v>1429</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>1434</v>
+        <v>1430</v>
       </c>
       <c r="B52" t="s">
-        <v>1435</v>
+        <v>1431</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.3">
@@ -8684,7 +8673,7 @@
         <v>1302</v>
       </c>
       <c r="B53" t="s">
-        <v>1436</v>
+        <v>1432</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.3">
@@ -8692,7 +8681,7 @@
         <v>1303</v>
       </c>
       <c r="B54" t="s">
-        <v>1437</v>
+        <v>1433</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.3">
@@ -8700,7 +8689,7 @@
         <v>1305</v>
       </c>
       <c r="B55" t="s">
-        <v>1438</v>
+        <v>1434</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.3">
@@ -8708,7 +8697,7 @@
         <v>1307</v>
       </c>
       <c r="B56" t="s">
-        <v>1439</v>
+        <v>1435</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.3">
@@ -8716,7 +8705,7 @@
         <v>1310</v>
       </c>
       <c r="B57" t="s">
-        <v>1440</v>
+        <v>1436</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.3">
@@ -8724,7 +8713,7 @@
         <v>1311</v>
       </c>
       <c r="B58" t="s">
-        <v>1439</v>
+        <v>1435</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.3">
@@ -8732,7 +8721,7 @@
         <v>1313</v>
       </c>
       <c r="B59" t="s">
-        <v>1438</v>
+        <v>1434</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.3">
@@ -8740,47 +8729,47 @@
         <v>1314</v>
       </c>
       <c r="B60" t="s">
-        <v>1441</v>
+        <v>1437</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>1442</v>
+        <v>1438</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>1443</v>
+        <v>1439</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>1444</v>
+        <v>1440</v>
       </c>
       <c r="B65" t="s">
-        <v>1445</v>
+        <v>1441</v>
       </c>
       <c r="C65" t="s">
-        <v>1446</v>
+        <v>1442</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>1447</v>
+        <v>1443</v>
       </c>
       <c r="B66" t="s">
-        <v>1448</v>
+        <v>1444</v>
       </c>
       <c r="C66" t="s">
-        <v>1449</v>
+        <v>1445</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>1450</v>
+        <v>1446</v>
       </c>
       <c r="B67" t="s">
-        <v>1451</v>
+        <v>1447</v>
       </c>
       <c r="C67" t="s">
         <v>792</v>
@@ -8788,10 +8777,10 @@
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>1452</v>
+        <v>1448</v>
       </c>
       <c r="B68" t="s">
-        <v>1453</v>
+        <v>1449</v>
       </c>
       <c r="C68" t="s">
         <v>798</v>
@@ -8799,17 +8788,17 @@
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>1454</v>
+        <v>1450</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>1455</v>
+        <v>1451</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>1432</v>
+        <v>1428</v>
       </c>
       <c r="B73" t="s">
         <v>5</v>
@@ -8996,90 +8985,90 @@
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
-        <v>1456</v>
+        <v>1452</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
-        <v>1457</v>
+        <v>1453</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
-        <v>1444</v>
+        <v>1440</v>
       </c>
       <c r="B88" t="s">
-        <v>1458</v>
+        <v>1454</v>
       </c>
       <c r="C88" t="s">
-        <v>1459</v>
+        <v>1455</v>
       </c>
       <c r="D88" t="s">
-        <v>1460</v>
+        <v>1456</v>
       </c>
       <c r="E88" t="s">
-        <v>1461</v>
+        <v>1457</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
-        <v>1447</v>
+        <v>1443</v>
       </c>
       <c r="B89" t="s">
-        <v>1462</v>
+        <v>1458</v>
       </c>
       <c r="C89" t="s">
-        <v>1463</v>
+        <v>1459</v>
       </c>
       <c r="D89" t="s">
-        <v>1464</v>
+        <v>1460</v>
       </c>
       <c r="E89" t="s">
-        <v>1465</v>
+        <v>1461</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
-        <v>1450</v>
+        <v>1446</v>
       </c>
       <c r="B90" t="s">
-        <v>1466</v>
+        <v>1462</v>
       </c>
       <c r="C90" t="s">
-        <v>1465</v>
+        <v>1461</v>
       </c>
       <c r="D90" t="s">
-        <v>1467</v>
+        <v>1463</v>
       </c>
       <c r="E90" t="s">
-        <v>1468</v>
+        <v>1464</v>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
-        <v>1452</v>
+        <v>1448</v>
       </c>
       <c r="B91" t="s">
-        <v>1469</v>
+        <v>1465</v>
       </c>
       <c r="C91" t="s">
-        <v>1464</v>
+        <v>1460</v>
       </c>
       <c r="D91" t="s">
-        <v>1470</v>
+        <v>1466</v>
       </c>
       <c r="E91" t="s">
-        <v>1471</v>
+        <v>1467</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
-        <v>1472</v>
+        <v>1468</v>
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
-        <v>1473</v>
+        <v>1469</v>
       </c>
       <c r="B94" t="s">
         <v>944</v>
@@ -9087,23 +9076,23 @@
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
-        <v>1474</v>
+        <v>1470</v>
       </c>
       <c r="B95" t="s">
-        <v>1475</v>
+        <v>1471</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
-        <v>1476</v>
+        <v>1472</v>
       </c>
       <c r="B96" t="s">
-        <v>1477</v>
+        <v>1473</v>
       </c>
     </row>
     <row r="98" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
-        <v>1478</v>
+        <v>1474</v>
       </c>
     </row>
   </sheetData>
@@ -9121,17 +9110,17 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>1479</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>1480</v>
+        <v>1476</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>1481</v>
+        <v>1477</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
@@ -9144,18 +9133,18 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>1482</v>
+        <v>1478</v>
       </c>
       <c r="B6" t="s">
-        <v>1483</v>
+        <v>1479</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>1484</v>
+        <v>1480</v>
       </c>
       <c r="B7" t="s">
-        <v>1485</v>
+        <v>1481</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
@@ -9163,23 +9152,23 @@
         <v>1300</v>
       </c>
       <c r="B8" t="s">
-        <v>1486</v>
+        <v>1482</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>1487</v>
+        <v>1483</v>
       </c>
       <c r="B9" t="s">
-        <v>1488</v>
+        <v>1484</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>1489</v>
+        <v>1485</v>
       </c>
       <c r="B10" t="s">
-        <v>1490</v>
+        <v>1486</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
@@ -9187,15 +9176,15 @@
         <v>823</v>
       </c>
       <c r="B11" t="s">
-        <v>1491</v>
+        <v>1487</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>1382</v>
+        <v>1378</v>
       </c>
       <c r="B12" t="s">
-        <v>1492</v>
+        <v>1488</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
@@ -9203,70 +9192,70 @@
         <v>1279</v>
       </c>
       <c r="B13" t="s">
-        <v>1493</v>
+        <v>1489</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>1494</v>
+        <v>1490</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>1495</v>
+        <v>1491</v>
       </c>
       <c r="B16" t="s">
-        <v>1496</v>
+        <v>1492</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>1497</v>
+        <v>1493</v>
       </c>
       <c r="B17" t="s">
-        <v>1498</v>
+        <v>1494</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>1499</v>
+        <v>1495</v>
       </c>
       <c r="B18" t="s">
-        <v>1500</v>
+        <v>1496</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>1389</v>
+        <v>1385</v>
       </c>
       <c r="B19" t="s">
-        <v>1501</v>
+        <v>1497</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>1391</v>
+        <v>1387</v>
       </c>
       <c r="B20" t="s">
-        <v>1502</v>
+        <v>1498</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>1393</v>
+        <v>1389</v>
       </c>
       <c r="B21" t="s">
-        <v>1503</v>
+        <v>1499</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>1504</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>1505</v>
+        <v>1501</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
@@ -9274,70 +9263,70 @@
         <v>944</v>
       </c>
       <c r="B26" t="s">
-        <v>1506</v>
+        <v>1502</v>
       </c>
       <c r="C26" t="s">
-        <v>1507</v>
+        <v>1503</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>1508</v>
+        <v>1504</v>
       </c>
       <c r="B27" t="s">
-        <v>1509</v>
+        <v>1505</v>
       </c>
       <c r="C27" t="s">
-        <v>1510</v>
+        <v>1506</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>1511</v>
+        <v>1507</v>
       </c>
       <c r="B28" t="s">
-        <v>1512</v>
+        <v>1508</v>
       </c>
       <c r="C28" t="s">
-        <v>1513</v>
+        <v>1509</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>1514</v>
+        <v>1510</v>
       </c>
       <c r="B29" t="s">
-        <v>1515</v>
+        <v>1511</v>
       </c>
       <c r="C29" t="s">
-        <v>1513</v>
+        <v>1509</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>1516</v>
+        <v>1512</v>
       </c>
       <c r="B30" t="s">
-        <v>1517</v>
+        <v>1513</v>
       </c>
       <c r="C30" t="s">
-        <v>1518</v>
+        <v>1514</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>1519</v>
+        <v>1515</v>
       </c>
       <c r="B31" t="s">
-        <v>1520</v>
+        <v>1516</v>
       </c>
       <c r="C31" t="s">
-        <v>1521</v>
+        <v>1517</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>1522</v>
+        <v>1518</v>
       </c>
       <c r="B32" t="s">
         <v>904</v>
@@ -9348,7 +9337,7 @@
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>1523</v>
+        <v>1519</v>
       </c>
       <c r="B33" t="s">
         <v>905</v>
@@ -9359,7 +9348,7 @@
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>1524</v>
+        <v>1520</v>
       </c>
       <c r="B34" t="s">
         <v>913</v>
@@ -9370,7 +9359,7 @@
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>1525</v>
+        <v>1521</v>
       </c>
       <c r="B35" t="s">
         <v>908</v>
@@ -9381,7 +9370,7 @@
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>1526</v>
+        <v>1522</v>
       </c>
       <c r="B36" t="s">
         <v>910</v>
@@ -9392,7 +9381,7 @@
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>1527</v>
+        <v>1523</v>
       </c>
       <c r="B37" t="s">
         <v>910</v>
@@ -9403,29 +9392,29 @@
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>1528</v>
+        <v>1524</v>
       </c>
       <c r="B38" t="s">
         <v>910</v>
       </c>
       <c r="C38" t="s">
-        <v>1529</v>
+        <v>1525</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>1530</v>
+        <v>1526</v>
       </c>
       <c r="B39" t="s">
         <v>910</v>
       </c>
       <c r="C39" t="s">
-        <v>1531</v>
+        <v>1527</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>1532</v>
+        <v>1528</v>
       </c>
       <c r="B40" t="s">
         <v>913</v>
@@ -9436,7 +9425,7 @@
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>1533</v>
+        <v>1529</v>
       </c>
       <c r="B41" t="s">
         <v>913</v>
@@ -9447,7 +9436,7 @@
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>1534</v>
+        <v>1530</v>
       </c>
       <c r="B42" t="s">
         <v>910</v>
@@ -9458,7 +9447,7 @@
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>1535</v>
+        <v>1531</v>
       </c>
       <c r="B43" t="s">
         <v>905</v>
@@ -9469,7 +9458,7 @@
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>1536</v>
+        <v>1532</v>
       </c>
       <c r="B44" t="s">
         <v>913</v>
@@ -9480,35 +9469,35 @@
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>1537</v>
+        <v>1533</v>
       </c>
       <c r="B45" t="s">
-        <v>1538</v>
+        <v>1534</v>
       </c>
       <c r="C45" t="s">
-        <v>1539</v>
+        <v>1535</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>1540</v>
+        <v>1536</v>
       </c>
       <c r="B46" t="s">
-        <v>1541</v>
+        <v>1537</v>
       </c>
       <c r="C46" t="s">
-        <v>1521</v>
+        <v>1517</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>1542</v>
+        <v>1538</v>
       </c>
       <c r="B48" t="s">
-        <v>1543</v>
+        <v>1539</v>
       </c>
       <c r="C48" t="s">
-        <v>1544</v>
+        <v>1540</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.3">
@@ -9516,32 +9505,32 @@
         <v>781</v>
       </c>
       <c r="B49" t="s">
-        <v>1545</v>
+        <v>1541</v>
       </c>
       <c r="C49" t="s">
-        <v>1546</v>
+        <v>1542</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>1547</v>
+        <v>1543</v>
       </c>
       <c r="B50" t="s">
-        <v>1548</v>
+        <v>1544</v>
       </c>
       <c r="C50" t="s">
-        <v>1549</v>
+        <v>1545</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>1550</v>
+        <v>1546</v>
       </c>
       <c r="B51" t="s">
-        <v>1551</v>
+        <v>1547</v>
       </c>
       <c r="C51" t="s">
-        <v>1552</v>
+        <v>1548</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.3">
@@ -9549,26 +9538,26 @@
         <v>823</v>
       </c>
       <c r="B52" t="s">
-        <v>1553</v>
+        <v>1549</v>
       </c>
       <c r="C52" t="s">
-        <v>1554</v>
+        <v>1550</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>1555</v>
+        <v>1551</v>
       </c>
       <c r="B54" t="s">
         <v>969</v>
       </c>
       <c r="C54" t="s">
-        <v>1556</v>
+        <v>1552</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>1557</v>
+        <v>1553</v>
       </c>
       <c r="B55" t="s">
         <v>939</v>
@@ -9579,7 +9568,7 @@
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>1558</v>
+        <v>1554</v>
       </c>
       <c r="B56" t="s">
         <v>920</v>
@@ -9590,10 +9579,10 @@
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>1559</v>
+        <v>1555</v>
       </c>
       <c r="B57" t="s">
-        <v>1560</v>
+        <v>1556</v>
       </c>
       <c r="C57" t="s">
         <v>905</v>
@@ -9601,40 +9590,40 @@
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>1561</v>
+        <v>1557</v>
       </c>
       <c r="B58" t="s">
-        <v>1560</v>
+        <v>1556</v>
       </c>
       <c r="C58" t="s">
-        <v>1560</v>
+        <v>1556</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>1562</v>
+        <v>1558</v>
       </c>
       <c r="B59" t="s">
-        <v>1560</v>
+        <v>1556</v>
       </c>
       <c r="C59" t="s">
-        <v>1560</v>
+        <v>1556</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>1563</v>
+        <v>1559</v>
       </c>
       <c r="B60" t="s">
-        <v>1560</v>
+        <v>1556</v>
       </c>
       <c r="C60" t="s">
-        <v>1560</v>
+        <v>1556</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>1564</v>
+        <v>1560</v>
       </c>
       <c r="B61" t="s">
         <v>940</v>
@@ -9645,36 +9634,36 @@
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>1565</v>
+        <v>1561</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>1566</v>
+        <v>1562</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>1567</v>
+        <v>1563</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>1568</v>
+        <v>1564</v>
       </c>
       <c r="B67" t="s">
         <v>969</v>
       </c>
       <c r="C67" t="s">
-        <v>1569</v>
+        <v>1565</v>
       </c>
       <c r="D67" t="s">
-        <v>1570</v>
+        <v>1566</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>1557</v>
+        <v>1553</v>
       </c>
       <c r="B68" t="s">
         <v>905</v>
@@ -9688,13 +9677,13 @@
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>1558</v>
+        <v>1554</v>
       </c>
       <c r="B69" t="s">
         <v>908</v>
       </c>
       <c r="C69" t="s">
-        <v>1571</v>
+        <v>1567</v>
       </c>
       <c r="D69" t="s">
         <v>1018</v>
@@ -9702,13 +9691,13 @@
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>1559</v>
+        <v>1555</v>
       </c>
       <c r="B70" t="s">
         <v>908</v>
       </c>
       <c r="C70" t="s">
-        <v>1572</v>
+        <v>1568</v>
       </c>
       <c r="D70" t="s">
         <v>1018</v>
@@ -9716,133 +9705,133 @@
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>1561</v>
+        <v>1557</v>
       </c>
       <c r="B71" t="s">
         <v>908</v>
       </c>
       <c r="C71" t="s">
-        <v>1573</v>
+        <v>1569</v>
       </c>
       <c r="D71" t="s">
-        <v>1574</v>
+        <v>1570</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>1562</v>
+        <v>1558</v>
       </c>
       <c r="B72" t="s">
         <v>908</v>
       </c>
       <c r="C72" t="s">
-        <v>1573</v>
+        <v>1569</v>
       </c>
       <c r="D72" t="s">
-        <v>1574</v>
+        <v>1570</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>1563</v>
+        <v>1559</v>
       </c>
       <c r="B73" t="s">
         <v>908</v>
       </c>
       <c r="C73" t="s">
-        <v>1573</v>
+        <v>1569</v>
       </c>
       <c r="D73" t="s">
-        <v>1574</v>
+        <v>1570</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
-        <v>1575</v>
+        <v>1571</v>
       </c>
       <c r="B74" t="s">
         <v>913</v>
       </c>
       <c r="C74" t="s">
-        <v>1576</v>
+        <v>1572</v>
       </c>
       <c r="D74" t="s">
-        <v>1577</v>
+        <v>1573</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>1578</v>
+        <v>1574</v>
       </c>
       <c r="B75" t="s">
         <v>913</v>
       </c>
       <c r="C75" t="s">
-        <v>1576</v>
+        <v>1572</v>
       </c>
       <c r="D75" t="s">
-        <v>1577</v>
+        <v>1573</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
-        <v>1579</v>
+        <v>1575</v>
       </c>
       <c r="B76" t="s">
         <v>913</v>
       </c>
       <c r="C76" t="s">
-        <v>1576</v>
+        <v>1572</v>
       </c>
       <c r="D76" t="s">
-        <v>1577</v>
+        <v>1573</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>1580</v>
+        <v>1576</v>
       </c>
       <c r="B77" t="s">
         <v>913</v>
       </c>
       <c r="C77" t="s">
-        <v>1581</v>
+        <v>1577</v>
       </c>
       <c r="D77" t="s">
-        <v>1582</v>
+        <v>1578</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
-        <v>1583</v>
+        <v>1579</v>
       </c>
       <c r="B78" t="s">
         <v>913</v>
       </c>
       <c r="C78" t="s">
-        <v>1584</v>
+        <v>1580</v>
       </c>
       <c r="D78" t="s">
-        <v>1585</v>
+        <v>1581</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
-        <v>1586</v>
+        <v>1582</v>
       </c>
       <c r="B79" t="s">
         <v>972</v>
       </c>
       <c r="C79" t="s">
-        <v>1576</v>
+        <v>1572</v>
       </c>
       <c r="D79" t="s">
-        <v>1587</v>
+        <v>1583</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
-        <v>1588</v>
+        <v>1584</v>
       </c>
       <c r="B80" t="s">
         <v>972</v>
@@ -9851,17 +9840,17 @@
         <v>972</v>
       </c>
       <c r="D80" t="s">
-        <v>1589</v>
+        <v>1585</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
-        <v>1590</v>
+        <v>1586</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
-        <v>1591</v>
+        <v>1587</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.3">
@@ -9872,88 +9861,88 @@
         <v>992</v>
       </c>
       <c r="C85" t="s">
-        <v>1592</v>
+        <v>1588</v>
       </c>
       <c r="D85" t="s">
-        <v>1593</v>
+        <v>1589</v>
       </c>
       <c r="E85" t="s">
-        <v>1594</v>
+        <v>1590</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
-        <v>1595</v>
+        <v>1591</v>
       </c>
       <c r="B86" t="s">
         <v>997</v>
       </c>
       <c r="C86" t="s">
-        <v>1596</v>
+        <v>1592</v>
       </c>
       <c r="D86" t="s">
         <v>910</v>
       </c>
       <c r="E86" t="s">
-        <v>1597</v>
+        <v>1593</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
-        <v>1598</v>
+        <v>1594</v>
       </c>
       <c r="B87" t="s">
-        <v>1599</v>
+        <v>1595</v>
       </c>
       <c r="C87" t="s">
-        <v>1600</v>
+        <v>1596</v>
       </c>
       <c r="D87" t="s">
         <v>1003</v>
       </c>
       <c r="E87" t="s">
-        <v>1601</v>
+        <v>1597</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
-        <v>1602</v>
+        <v>1598</v>
       </c>
       <c r="B88" t="s">
-        <v>1603</v>
+        <v>1599</v>
       </c>
       <c r="C88" t="s">
-        <v>1604</v>
+        <v>1600</v>
       </c>
       <c r="D88" t="s">
         <v>984</v>
       </c>
       <c r="E88" t="s">
-        <v>1605</v>
+        <v>1601</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
-        <v>1606</v>
+        <v>1602</v>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
-        <v>1607</v>
+        <v>1603</v>
       </c>
       <c r="B91" t="s">
         <v>969</v>
       </c>
       <c r="C91" t="s">
-        <v>1569</v>
+        <v>1565</v>
       </c>
       <c r="D91" t="s">
-        <v>1570</v>
+        <v>1566</v>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
-        <v>1557</v>
+        <v>1553</v>
       </c>
       <c r="B92" t="s">
         <v>1012</v>
@@ -9967,7 +9956,7 @@
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
-        <v>1558</v>
+        <v>1554</v>
       </c>
       <c r="B93" t="s">
         <v>972</v>
@@ -9981,7 +9970,7 @@
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
-        <v>1559</v>
+        <v>1555</v>
       </c>
       <c r="B94" t="s">
         <v>908</v>
@@ -9995,7 +9984,7 @@
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
-        <v>1561</v>
+        <v>1557</v>
       </c>
       <c r="B95" t="s">
         <v>1017</v>
@@ -10009,7 +9998,7 @@
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
-        <v>1562</v>
+        <v>1558</v>
       </c>
       <c r="B96" t="s">
         <v>1019</v>
@@ -10023,7 +10012,7 @@
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
-        <v>1563</v>
+        <v>1559</v>
       </c>
       <c r="B97" t="s">
         <v>908</v>
@@ -10037,7 +10026,7 @@
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
-        <v>1583</v>
+        <v>1579</v>
       </c>
       <c r="B98" t="s">
         <v>984</v>
@@ -10051,7 +10040,7 @@
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
-        <v>1586</v>
+        <v>1582</v>
       </c>
       <c r="B99" t="s">
         <v>972</v>
@@ -10065,21 +10054,21 @@
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
-        <v>1608</v>
+        <v>1604</v>
       </c>
       <c r="B101" t="s">
         <v>969</v>
       </c>
       <c r="C101" t="s">
-        <v>1569</v>
+        <v>1565</v>
       </c>
       <c r="D101" t="s">
-        <v>1570</v>
+        <v>1566</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
-        <v>1557</v>
+        <v>1553</v>
       </c>
       <c r="B102" t="s">
         <v>1013</v>
@@ -10093,7 +10082,7 @@
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
-        <v>1558</v>
+        <v>1554</v>
       </c>
       <c r="B103" t="s">
         <v>972</v>
@@ -10102,26 +10091,26 @@
         <v>1026</v>
       </c>
       <c r="D103" t="s">
-        <v>1609</v>
+        <v>1605</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
-        <v>1559</v>
+        <v>1555</v>
       </c>
       <c r="B104" t="s">
         <v>1015</v>
       </c>
       <c r="C104" t="s">
-        <v>1610</v>
+        <v>1606</v>
       </c>
       <c r="D104" t="s">
-        <v>1610</v>
+        <v>1606</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
-        <v>1561</v>
+        <v>1557</v>
       </c>
       <c r="B105" t="s">
         <v>1018</v>
@@ -10130,12 +10119,12 @@
         <v>1028</v>
       </c>
       <c r="D105" t="s">
-        <v>1611</v>
+        <v>1607</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
-        <v>1562</v>
+        <v>1558</v>
       </c>
       <c r="B106" t="s">
         <v>1018</v>
@@ -10144,12 +10133,12 @@
         <v>1028</v>
       </c>
       <c r="D106" t="s">
-        <v>1611</v>
+        <v>1607</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
-        <v>1563</v>
+        <v>1559</v>
       </c>
       <c r="B107" t="s">
         <v>1020</v>
@@ -10158,12 +10147,12 @@
         <v>1030</v>
       </c>
       <c r="D107" t="s">
-        <v>1612</v>
+        <v>1608</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
-        <v>1580</v>
+        <v>1576</v>
       </c>
       <c r="B108" t="s">
         <v>1022</v>
@@ -10177,7 +10166,7 @@
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
-        <v>1583</v>
+        <v>1579</v>
       </c>
       <c r="B109" t="s">
         <v>1023</v>
@@ -10186,26 +10175,26 @@
         <v>1033</v>
       </c>
       <c r="D109" t="s">
-        <v>1613</v>
+        <v>1609</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
-        <v>1586</v>
+        <v>1582</v>
       </c>
       <c r="B110" t="s">
         <v>1024</v>
       </c>
       <c r="C110" t="s">
-        <v>1614</v>
+        <v>1610</v>
       </c>
       <c r="D110" t="s">
-        <v>1560</v>
+        <v>1556</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
-        <v>1588</v>
+        <v>1584</v>
       </c>
       <c r="B111" t="s">
         <v>972</v>
@@ -10219,21 +10208,21 @@
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
-        <v>1615</v>
+        <v>1611</v>
       </c>
       <c r="B113" t="s">
         <v>969</v>
       </c>
       <c r="C113" t="s">
-        <v>1569</v>
+        <v>1565</v>
       </c>
       <c r="D113" t="s">
-        <v>1570</v>
+        <v>1566</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
-        <v>1557</v>
+        <v>1553</v>
       </c>
       <c r="B114" t="s">
         <v>1014</v>
@@ -10247,133 +10236,133 @@
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
-        <v>1558</v>
+        <v>1554</v>
       </c>
       <c r="B115" t="s">
         <v>972</v>
       </c>
       <c r="C115" t="s">
-        <v>1616</v>
+        <v>1612</v>
       </c>
       <c r="D115" t="s">
-        <v>1617</v>
+        <v>1613</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
-        <v>1559</v>
+        <v>1555</v>
       </c>
       <c r="B116" t="s">
         <v>1016</v>
       </c>
       <c r="C116" t="s">
-        <v>1618</v>
+        <v>1614</v>
       </c>
       <c r="D116" t="s">
-        <v>1619</v>
+        <v>1615</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
-        <v>1561</v>
+        <v>1557</v>
       </c>
       <c r="B117" t="s">
         <v>1016</v>
       </c>
       <c r="C117" t="s">
-        <v>1620</v>
+        <v>1616</v>
       </c>
       <c r="D117" t="s">
-        <v>1621</v>
+        <v>1617</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
-        <v>1562</v>
+        <v>1558</v>
       </c>
       <c r="B118" t="s">
         <v>1016</v>
       </c>
       <c r="C118" t="s">
-        <v>1620</v>
+        <v>1616</v>
       </c>
       <c r="D118" t="s">
-        <v>1621</v>
+        <v>1617</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
-        <v>1563</v>
+        <v>1559</v>
       </c>
       <c r="B119" t="s">
         <v>1021</v>
       </c>
       <c r="C119" t="s">
-        <v>1622</v>
+        <v>1618</v>
       </c>
       <c r="D119" t="s">
-        <v>1623</v>
+        <v>1619</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
-        <v>1580</v>
+        <v>1576</v>
       </c>
       <c r="B120" t="s">
         <v>1021</v>
       </c>
       <c r="C120" t="s">
-        <v>1622</v>
+        <v>1618</v>
       </c>
       <c r="D120" t="s">
-        <v>1623</v>
+        <v>1619</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
-        <v>1583</v>
+        <v>1579</v>
       </c>
       <c r="B121" t="s">
-        <v>1624</v>
+        <v>1620</v>
       </c>
       <c r="C121" t="s">
-        <v>1625</v>
+        <v>1621</v>
       </c>
       <c r="D121" t="s">
-        <v>1573</v>
+        <v>1569</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
-        <v>1586</v>
+        <v>1582</v>
       </c>
       <c r="B122" t="s">
-        <v>1626</v>
+        <v>1622</v>
       </c>
       <c r="C122" t="s">
-        <v>1622</v>
+        <v>1618</v>
       </c>
       <c r="D122" t="s">
-        <v>1627</v>
+        <v>1623</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
-        <v>1564</v>
+        <v>1560</v>
       </c>
       <c r="B123" t="s">
-        <v>1628</v>
+        <v>1624</v>
       </c>
       <c r="C123" t="s">
-        <v>1622</v>
+        <v>1618</v>
       </c>
       <c r="D123" t="s">
-        <v>1623</v>
+        <v>1619</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
-        <v>1588</v>
+        <v>1584</v>
       </c>
       <c r="B124" t="s">
         <v>972</v>
@@ -10387,20 +10376,20 @@
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
-        <v>1629</v>
+        <v>1625</v>
       </c>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
-        <v>1630</v>
+        <v>1626</v>
       </c>
     </row>
     <row r="129" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
-        <v>1444</v>
+        <v>1440</v>
       </c>
       <c r="B129" t="s">
-        <v>1631</v>
+        <v>1627</v>
       </c>
       <c r="C129" t="s">
         <v>806</v>
@@ -10411,100 +10400,100 @@
     </row>
     <row r="130" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
-        <v>1447</v>
+        <v>1443</v>
       </c>
       <c r="B130" t="s">
-        <v>1632</v>
+        <v>1628</v>
       </c>
       <c r="C130" t="s">
-        <v>1633</v>
+        <v>1629</v>
       </c>
       <c r="D130" t="s">
-        <v>1634</v>
+        <v>1630</v>
       </c>
     </row>
     <row r="131" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
-        <v>1450</v>
+        <v>1446</v>
       </c>
       <c r="B131" t="s">
-        <v>1635</v>
+        <v>1631</v>
       </c>
       <c r="C131" t="s">
-        <v>1636</v>
+        <v>1632</v>
       </c>
       <c r="D131" t="s">
-        <v>1637</v>
+        <v>1633</v>
       </c>
     </row>
     <row r="132" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
-        <v>1452</v>
+        <v>1448</v>
       </c>
       <c r="B132" t="s">
-        <v>1638</v>
+        <v>1634</v>
       </c>
       <c r="C132" t="s">
-        <v>1639</v>
+        <v>1635</v>
       </c>
       <c r="D132" t="s">
-        <v>1640</v>
+        <v>1636</v>
       </c>
     </row>
     <row r="134" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
-        <v>1641</v>
+        <v>1637</v>
       </c>
     </row>
     <row r="136" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
-        <v>1642</v>
+        <v>1638</v>
       </c>
     </row>
     <row r="137" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
-        <v>1643</v>
+        <v>1639</v>
       </c>
     </row>
     <row r="138" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
+        <v>1640</v>
+      </c>
+      <c r="B138" t="s">
+        <v>1641</v>
+      </c>
+      <c r="C138" t="s">
+        <v>1642</v>
+      </c>
+      <c r="D138" t="s">
+        <v>1643</v>
+      </c>
+      <c r="E138" t="s">
         <v>1644</v>
       </c>
-      <c r="B138" t="s">
+      <c r="F138" t="s">
         <v>1645</v>
       </c>
-      <c r="C138" t="s">
+      <c r="G138" t="s">
         <v>1646</v>
       </c>
-      <c r="D138" t="s">
+      <c r="H138" t="s">
         <v>1647</v>
       </c>
-      <c r="E138" t="s">
+      <c r="I138" t="s">
         <v>1648</v>
       </c>
-      <c r="F138" t="s">
+      <c r="J138" t="s">
         <v>1649</v>
       </c>
-      <c r="G138" t="s">
+      <c r="K138" t="s">
         <v>1650</v>
       </c>
-      <c r="H138" t="s">
+      <c r="L138" t="s">
         <v>1651</v>
       </c>
-      <c r="I138" t="s">
+      <c r="M138" t="s">
         <v>1652</v>
-      </c>
-      <c r="J138" t="s">
-        <v>1653</v>
-      </c>
-      <c r="K138" t="s">
-        <v>1654</v>
-      </c>
-      <c r="L138" t="s">
-        <v>1655</v>
-      </c>
-      <c r="M138" t="s">
-        <v>1656</v>
       </c>
     </row>
     <row r="139" spans="1:13" x14ac:dyDescent="0.3">
@@ -12969,80 +12958,80 @@
     </row>
     <row r="200" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A200" t="s">
-        <v>1657</v>
+        <v>1653</v>
       </c>
     </row>
     <row r="202" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A202" t="s">
-        <v>1457</v>
+        <v>1453</v>
       </c>
     </row>
     <row r="203" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A203" t="s">
-        <v>1444</v>
+        <v>1440</v>
       </c>
       <c r="B203" t="s">
-        <v>1458</v>
+        <v>1454</v>
       </c>
       <c r="C203" t="s">
-        <v>1459</v>
+        <v>1455</v>
       </c>
       <c r="D203" t="s">
-        <v>1460</v>
+        <v>1456</v>
       </c>
       <c r="E203" t="s">
-        <v>1461</v>
+        <v>1457</v>
       </c>
     </row>
     <row r="204" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A204" t="s">
-        <v>1447</v>
+        <v>1443</v>
       </c>
       <c r="B204" t="s">
-        <v>1462</v>
+        <v>1458</v>
       </c>
       <c r="C204" t="s">
-        <v>1463</v>
+        <v>1459</v>
       </c>
       <c r="D204" t="s">
-        <v>1464</v>
+        <v>1460</v>
       </c>
       <c r="E204" t="s">
-        <v>1465</v>
+        <v>1461</v>
       </c>
     </row>
     <row r="205" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A205" t="s">
-        <v>1450</v>
+        <v>1446</v>
       </c>
       <c r="B205" t="s">
-        <v>1466</v>
+        <v>1462</v>
       </c>
       <c r="C205" t="s">
-        <v>1465</v>
+        <v>1461</v>
       </c>
       <c r="D205" t="s">
-        <v>1467</v>
+        <v>1463</v>
       </c>
       <c r="E205" t="s">
-        <v>1468</v>
+        <v>1464</v>
       </c>
     </row>
     <row r="206" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A206" t="s">
-        <v>1452</v>
+        <v>1448</v>
       </c>
       <c r="B206" t="s">
-        <v>1469</v>
+        <v>1465</v>
       </c>
       <c r="C206" t="s">
-        <v>1464</v>
+        <v>1460</v>
       </c>
       <c r="D206" t="s">
-        <v>1470</v>
+        <v>1466</v>
       </c>
       <c r="E206" t="s">
-        <v>1471</v>
+        <v>1467</v>
       </c>
     </row>
   </sheetData>
@@ -14836,12 +14825,6 @@
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="B29:B31"/>
-    <mergeCell ref="B14:B16"/>
-    <mergeCell ref="A8:A10"/>
-    <mergeCell ref="A26:A28"/>
-    <mergeCell ref="A17:A19"/>
-    <mergeCell ref="A20:A22"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A5:A7"/>
     <mergeCell ref="A23:A25"/>
@@ -14858,6 +14841,12 @@
     <mergeCell ref="B17:B19"/>
     <mergeCell ref="B23:B25"/>
     <mergeCell ref="A29:A31"/>
+    <mergeCell ref="B29:B31"/>
+    <mergeCell ref="B14:B16"/>
+    <mergeCell ref="A8:A10"/>
+    <mergeCell ref="A26:A28"/>
+    <mergeCell ref="A17:A19"/>
+    <mergeCell ref="A20:A22"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <ignoredErrors>
@@ -15752,10 +15741,10 @@
         <v>493</v>
       </c>
       <c r="F41" t="s">
-        <v>1658</v>
+        <v>1654</v>
       </c>
       <c r="G41" t="s">
-        <v>1659</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Gate CRYSTAWOLF-BASTION's counter-attack and stun chance behind HP<50%
The previous rework applied the counter-attack (and its stun chance) every
round regardless of HP. Correct intent: HP>50% only grants ATK+25% (no
counter/stun); HP<50% grants DEF+25% plus the guaranteed counter and 10%
stun-on-hit chance. Verified via 30 trials that neither counter nor stun
ever fire while HP>50%. Synced SYMBEAST_Evolve_Forms.xlsx.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SYMBEAST_Evolve_Forms.xlsx
+++ b/SYMBEAST_Evolve_Forms.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\skyit\Desktop\Symbeast-main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EF239C5-A0BE-42C2-83F7-E4C449AD9C46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EE5C70A-802E-4FF3-93D9-8F61F65F94A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5000,7 +5000,7 @@
     <t>โจมตี ×2.0 ทะลุ DEF ทั้งหมด + สะท้อนดาเมจทั้งหมดเทิร์นนี้ จากนั้นสะท้อน 50% และลดดาเมจที่รับ 15% นาน 3 เทิร์น</t>
   </si>
   <si>
-    <t>เมื่อ HP &gt; 50%: ATK+25% เมื่อ HP &lt; 50%: DEF+25% โต้กลับด้วยดาเมจ 75% ทุกรอบ และเมื่อโดนโจมตีมีโอกาส 10% ทำให้ศัตรูสต้น</t>
+    <t>เมื่อ HP &gt; 50%: ATK+25% เมื่อ HP &lt; 50%: DEF+25% โต้กลับด้วยดาเมจ 75% ทุกรอบ และมีโอกาส 10% ทำให้ศัตรูสต้นเมื่อโดนโจมตี</t>
   </si>
 </sst>
 </file>
@@ -14829,12 +14829,6 @@
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="B29:B31"/>
-    <mergeCell ref="B14:B16"/>
-    <mergeCell ref="A8:A10"/>
-    <mergeCell ref="A26:A28"/>
-    <mergeCell ref="A17:A19"/>
-    <mergeCell ref="A20:A22"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A5:A7"/>
     <mergeCell ref="A23:A25"/>
@@ -14851,6 +14845,12 @@
     <mergeCell ref="B17:B19"/>
     <mergeCell ref="B23:B25"/>
     <mergeCell ref="A29:A31"/>
+    <mergeCell ref="B29:B31"/>
+    <mergeCell ref="B14:B16"/>
+    <mergeCell ref="A8:A10"/>
+    <mergeCell ref="A26:A28"/>
+    <mergeCell ref="A17:A19"/>
+    <mergeCell ref="A20:A22"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <ignoredErrors>

</xml_diff>

<commit_message>
Design Fusion Passives (proposal, not yet implemented)
Adds two Excel sheets exploring a Fusion mechanic (2 pets -> Fusion Egg ->
inherited bonus passive): "Fusion Passives" (55 per-pair designs) and
"Fusion Passives v2" (40 half-strength "Echo" variants, one per Evolve II
form, chosen approach). Design-only, no game code changes yet.
</commit_message>
<xml_diff>
--- a/SYMBEAST_Evolve_Forms.xlsx
+++ b/SYMBEAST_Evolve_Forms.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\skyit\Desktop\Symbeast-main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73699FB6-166A-4DFB-B66A-C717A868DC6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2068D9C-48DA-419B-8811-7E187A3DE873}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="10" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Evolved Forms" sheetId="1" r:id="rId1"/>
@@ -27,13 +27,15 @@
     <sheet name="Raid Rewards" sheetId="12" r:id="rId12"/>
     <sheet name="Tower Rewards" sheetId="13" r:id="rId13"/>
     <sheet name="Scout Rewards" sheetId="14" r:id="rId14"/>
+    <sheet name="Fusion Passives" sheetId="15" r:id="rId15"/>
+    <sheet name="Fusion Passives v2" sheetId="16" r:id="rId16"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2601" uniqueCount="1656">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3203" uniqueCount="1991">
   <si>
     <t>SYMBEAST — Evolved Forms (Stage 1, 10 forms)</t>
   </si>
@@ -5001,6 +5003,1011 @@
   </si>
   <si>
     <t>15% โอกาสทำให้ศัตรูติดเผาไหม้เมื่อโจมตีโดน</t>
+  </si>
+  <si>
+    <t>SYMBEAST — Fusion Passives (proposal, ยังไม่ implement) — Fuse 2 Evolved-stage pets -&gt; Fusion Egg -&gt; hatch normally -&gt; pet carries 1 inherited passive slot</t>
+  </si>
+  <si>
+    <t>Category | Parent 1 | Parent 2 | Icon | Name | Effect (EN) | Effect (TH)</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Parent 1</t>
+  </si>
+  <si>
+    <t>Parent 2</t>
+  </si>
+  <si>
+    <t>Pure-blood</t>
+  </si>
+  <si>
+    <t>💢</t>
+  </si>
+  <si>
+    <t>RAGE BLOOD</t>
+  </si>
+  <si>
+    <t>On each WIN, ATK +10% (stacks up to 3 times)</t>
+  </si>
+  <si>
+    <t>ทุกครั้งที่ WIN, ATK+10% สะสม (สูงสุด 3 ครั้ง)</t>
+  </si>
+  <si>
+    <t>🐼</t>
+  </si>
+  <si>
+    <t>TWIN FANG</t>
+  </si>
+  <si>
+    <t>On crit, 10% chance to strike again immediately for 50% damage</t>
+  </si>
+  <si>
+    <t>คริติคอลแล้ว 10% โอกาสโจมตีซ้ำทันที (ดาเมจ 50%)</t>
+  </si>
+  <si>
+    <t>🩸</t>
+  </si>
+  <si>
+    <t>CRIMSON CORE</t>
+  </si>
+  <si>
+    <t>Lifesteal is doubled while HP &lt; 50%</t>
+  </si>
+  <si>
+    <t>ดูดเลือดที่ได้ ×2 เมื่อ HP&lt;50%</t>
+  </si>
+  <si>
+    <t>CHAIN LIGHTNING</t>
+  </si>
+  <si>
+    <t>When you stun the enemy, 20% chance to stun them again next round</t>
+  </si>
+  <si>
+    <t>สตันติดแล้ว มีโอกาส 20% สตันต่ออีกเทิร์น</t>
+  </si>
+  <si>
+    <t>🏆</t>
+  </si>
+  <si>
+    <t>GRAND CHAMPION</t>
+  </si>
+  <si>
+    <t>Win 2 rounds in a row: permanent ATK+30% for the rest of the battle (once)</t>
+  </si>
+  <si>
+    <t>ชนะ 2 รอบติด ATK+30% ถาวรตลอดการต่อสู้ (ครั้งเดียว)</t>
+  </si>
+  <si>
+    <t>🗿</t>
+  </si>
+  <si>
+    <t>STONE BLOOD</t>
+  </si>
+  <si>
+    <t>Every 3 turns, 20% chance to fully block all damage (100%)</t>
+  </si>
+  <si>
+    <t>ทุก 3 เทิร์น 20% โอกาสบล็อกดาเมจเต็ม 100%</t>
+  </si>
+  <si>
+    <t>👻</t>
+  </si>
+  <si>
+    <t>GHOST BLOOD</t>
+  </si>
+  <si>
+    <t>After a successful dodge, the next attack is a guaranteed crit</t>
+  </si>
+  <si>
+    <t>หลบสำเร็จแล้ว โจมตีถัดไปคริติคอลการันตี</t>
+  </si>
+  <si>
+    <t>🌪️</t>
+  </si>
+  <si>
+    <t>ETERNAL GUARD</t>
+  </si>
+  <si>
+    <t>On a successful dodge, heal an extra 10% Max HP (total 25%)</t>
+  </si>
+  <si>
+    <t>หลบสำเร็จ ฟื้น HP เพิ่มอีก 10% (รวม 25%)</t>
+  </si>
+  <si>
+    <t>🦅</t>
+  </si>
+  <si>
+    <t>SKYFORT</t>
+  </si>
+  <si>
+    <t>Both on WIN and LOSE, reduce damage taken by an extra 10%</t>
+  </si>
+  <si>
+    <t>WIN และ LOSE ลดดาเมจเพิ่มอีก 10% ทั้ง 2 กรณี</t>
+  </si>
+  <si>
+    <t>ABSOLUTE WALL</t>
+  </si>
+  <si>
+    <t>When the damage-halving effect triggers, reduce the remaining damage by another 10%</t>
+  </si>
+  <si>
+    <t>ลดดาเมจสำเร็จ (halve) ดาเมจที่เหลือ -10% เพิ่ม</t>
+  </si>
+  <si>
+    <t>Cross-blood</t>
+  </si>
+  <si>
+    <t>🔥</t>
+  </si>
+  <si>
+    <t>BERSERK FOCUS</t>
+  </si>
+  <si>
+    <t>On crit, ATK+15% stacking for the rest of the battle</t>
+  </si>
+  <si>
+    <t>คริติคอลแล้ว ATK+15% สะสมตลอดการต่อสู้</t>
+  </si>
+  <si>
+    <t>💪</t>
+  </si>
+  <si>
+    <t>BLOODRAGE</t>
+  </si>
+  <si>
+    <t>Lifesteal gained is converted into permanent ATK +5% per proc (stacks)</t>
+  </si>
+  <si>
+    <t>ดูดเลือดที่ได้ เปลี่ยนเป็น ATK ถาวร +5%/ครั้ง (สะสมได้)</t>
+  </si>
+  <si>
+    <t>THUNDER FIST</t>
+  </si>
+  <si>
+    <t>On WIN, 20% chance to stun the enemy</t>
+  </si>
+  <si>
+    <t>WIN แล้ว 20% โอกาสสตันศัตรู</t>
+  </si>
+  <si>
+    <t>🥊</t>
+  </si>
+  <si>
+    <t>RISING FIST</t>
+  </si>
+  <si>
+    <t>Win 3 rounds in a row: permanent ATK+50% (once per battle)</t>
+  </si>
+  <si>
+    <t>ชนะ 3 รอบติด ATK+50% ถาวร (ครั้งเดียว/battle)</t>
+  </si>
+  <si>
+    <t>UNSTOPPABLE WALL</t>
+  </si>
+  <si>
+    <t>15% chance to counter-attack for 50% damage when hit</t>
+  </si>
+  <si>
+    <t>15% โอกาสโต้กลับดาเมจ 50% เมื่อถูกโจมตี</t>
+  </si>
+  <si>
+    <t>👊</t>
+  </si>
+  <si>
+    <t>PHANTOM FIST</t>
+  </si>
+  <si>
+    <t>15% chance to dodge and counter-attack for 75% damage</t>
+  </si>
+  <si>
+    <t>15% โอกาสหลบ พร้อมโจมตีสวนกลับดาเมจ 75%</t>
+  </si>
+  <si>
+    <t>🦶</t>
+  </si>
+  <si>
+    <t>SWIFT FIST</t>
+  </si>
+  <si>
+    <t>10% chance to dodge, with ATK+15% next round</t>
+  </si>
+  <si>
+    <t>10% โอกาสหลบ พร้อม ATK+15% เทิร์นถัดไป</t>
+  </si>
+  <si>
+    <t>AERIAL BRUISER</t>
+  </si>
+  <si>
+    <t>On WIN, ATK+20% and damage taken -15% that round</t>
+  </si>
+  <si>
+    <t>WIN: ATK+20% และรับดาเมจ-15% รอบนั้น</t>
+  </si>
+  <si>
+    <t>🗻</t>
+  </si>
+  <si>
+    <t>JUGGERNAUT</t>
+  </si>
+  <si>
+    <t>Every 3 turns, deal +50% damage on that attack once</t>
+  </si>
+  <si>
+    <t>ทุก 3 เทิร์น โจมตีดาเมจ+50% ครั้งเดียว</t>
+  </si>
+  <si>
+    <t>CRIMSON STRIKE</t>
+  </si>
+  <si>
+    <t>On crit, lifesteal 30% of the damage dealt</t>
+  </si>
+  <si>
+    <t>คริติคอลแล้ว ดูดเลือด 30% ของดาเมจที่สร้าง</t>
+  </si>
+  <si>
+    <t>FLASH CRIT</t>
+  </si>
+  <si>
+    <t>On crit, 25% chance to instantly stun the enemy</t>
+  </si>
+  <si>
+    <t>คริติคอลแล้ว 25% โอกาสสตันศัตรูทันที</t>
+  </si>
+  <si>
+    <t>🎯</t>
+  </si>
+  <si>
+    <t>CHAMPION'S EYE</t>
+  </si>
+  <si>
+    <t>On WIN, crit chance +15% next round</t>
+  </si>
+  <si>
+    <t>WIN: โอกาสคริติคอล+15% รอบถัดไป</t>
+  </si>
+  <si>
+    <t>🪨</t>
+  </si>
+  <si>
+    <t>IRON CRIT</t>
+  </si>
+  <si>
+    <t>On crit, damage taken -20% next round</t>
+  </si>
+  <si>
+    <t>คริติคอลแล้ว รับดาเมจ-20% เทิร์นถัดไป</t>
+  </si>
+  <si>
+    <t>🥷</t>
+  </si>
+  <si>
+    <t>SHADOW CRIT</t>
+  </si>
+  <si>
+    <t>On a successful dodge, crit chance +30% next attack</t>
+  </si>
+  <si>
+    <t>หลบสำเร็จ โจมตีถัดไปคริ+30%</t>
+  </si>
+  <si>
+    <t>🌀</t>
+  </si>
+  <si>
+    <t>CRITICAL GUARD</t>
+  </si>
+  <si>
+    <t>On a successful dodge, heal 10% HP with crit chance +10%</t>
+  </si>
+  <si>
+    <t>หลบสำเร็จ ฟื้น HP 10% พร้อมคริ+10%</t>
+  </si>
+  <si>
+    <t>SKY CRIT</t>
+  </si>
+  <si>
+    <t>On WIN, guaranteed crit x2.0 that round</t>
+  </si>
+  <si>
+    <t>WIN: คริติคอล ×2.0 การันตีเทิร์นนั้น</t>
+  </si>
+  <si>
+    <t>GUARDIAN CRIT</t>
+  </si>
+  <si>
+    <t>When the damage-halving effect triggers, next attack is a guaranteed crit</t>
+  </si>
+  <si>
+    <t>ลดดาเมจสำเร็จ โจมตีถัดไปคริการันตี</t>
+  </si>
+  <si>
+    <t>🦷</t>
+  </si>
+  <si>
+    <t>VENOM FANG</t>
+  </si>
+  <si>
+    <t>On a successful lifesteal, 15% chance to stun the enemy</t>
+  </si>
+  <si>
+    <t>ดูดเลือดสำเร็จ 15% โอกาสสตันศัตรู</t>
+  </si>
+  <si>
+    <t>VICTOR'S BITE</t>
+  </si>
+  <si>
+    <t>On WIN, lifesteal increases to 40% of damage dealt</t>
+  </si>
+  <si>
+    <t>WIN: ดูดเลือดเพิ่มเป็น 40% ของดาเมจ</t>
+  </si>
+  <si>
+    <t>🔄</t>
+  </si>
+  <si>
+    <t>VAMPIRIC WALL</t>
+  </si>
+  <si>
+    <t>Reflected damage converts half of itself into HP healed</t>
+  </si>
+  <si>
+    <t>สะท้อนดาเมจ เปลี่ยนครึ่งหนึ่งเป็นฟื้น HP</t>
+  </si>
+  <si>
+    <t>🐺</t>
+  </si>
+  <si>
+    <t>PHANTOM FANGS</t>
+  </si>
+  <si>
+    <t>15% chance to lifesteal 50% of damage dealt and dodge that same turn</t>
+  </si>
+  <si>
+    <t>15% โอกาสดูดเลือด 50% พร้อมหลบเทิร์นนั้น</t>
+  </si>
+  <si>
+    <t>DRAIN STEP</t>
+  </si>
+  <si>
+    <t>On a successful dodge, instantly lifesteal 15% Max HP</t>
+  </si>
+  <si>
+    <t>หลบสำเร็จ ดูดเลือด 15% MaxHP ทันที</t>
+  </si>
+  <si>
+    <t>BLOOD WING</t>
+  </si>
+  <si>
+    <t>On WIN, lifesteal an extra +15% on top of the base amount</t>
+  </si>
+  <si>
+    <t>WIN: ดูดเลือดเพิ่ม+15% จากที่มีอยู่</t>
+  </si>
+  <si>
+    <t>STONE FANG</t>
+  </si>
+  <si>
+    <t>When the damage-halving effect triggers, lifesteal 20% of the damage reduced</t>
+  </si>
+  <si>
+    <t>ลดดาเมจสำเร็จ ดูดเลือด 20% ของดาเมจที่ลดได้</t>
+  </si>
+  <si>
+    <t>VICTORY SHOCK</t>
+  </si>
+  <si>
+    <t>On WIN, 25% chance to instantly stun the enemy</t>
+  </si>
+  <si>
+    <t>WIN: 25% โอกาสสตันศัตรูทันที</t>
+  </si>
+  <si>
+    <t>STATIC WALL</t>
+  </si>
+  <si>
+    <t>When you reflect damage, 15% chance to also stun the enemy</t>
+  </si>
+  <si>
+    <t>สะท้อนดาเมจ 15% โอกาสสตันติดไปด้วย</t>
+  </si>
+  <si>
+    <t>GHOST BOLT</t>
+  </si>
+  <si>
+    <t>After a successful stun, automatically dodge the enemy's next attack</t>
+  </si>
+  <si>
+    <t>สตันสำเร็จ หลบการโจมตีเทิร์นถัดไปอัตโนมัติ</t>
+  </si>
+  <si>
+    <t>QUICK SHOCK</t>
+  </si>
+  <si>
+    <t>On a successful dodge, 20% chance to stun the enemy back</t>
+  </si>
+  <si>
+    <t>หลบสำเร็จ 20% โอกาสสตันศัตรูสวน</t>
+  </si>
+  <si>
+    <t>STORM WING</t>
+  </si>
+  <si>
+    <t>On WIN, SPD+30% next round</t>
+  </si>
+  <si>
+    <t>WIN: SPD+30% เทิร์นถัดไป</t>
+  </si>
+  <si>
+    <t>THUNDER WALL</t>
+  </si>
+  <si>
+    <t>When the damage-halving effect triggers, 20% chance to stun the enemy</t>
+  </si>
+  <si>
+    <t>ลดดาเมจสำเร็จ 20% โอกาสสตันศัตรู</t>
+  </si>
+  <si>
+    <t>UNBREAKABLE</t>
+  </si>
+  <si>
+    <t>On WIN, reflect an extra 30% damage that round</t>
+  </si>
+  <si>
+    <t>WIN: สะท้อนดาเมจเพิ่ม 30% รอบนั้น</t>
+  </si>
+  <si>
+    <t>👑</t>
+  </si>
+  <si>
+    <t>PHANTOM VICTOR</t>
+  </si>
+  <si>
+    <t>On WIN, fully dodge the enemy's next attack (100%)</t>
+  </si>
+  <si>
+    <t>WIN: หลบการโจมตีรอบถัดไป 100%</t>
+  </si>
+  <si>
+    <t>🏅</t>
+  </si>
+  <si>
+    <t>SWIFT VICTORY</t>
+  </si>
+  <si>
+    <t>On WIN, instantly heal 15% HP</t>
+  </si>
+  <si>
+    <t>WIN: ฟื้น HP 15% ทันที</t>
+  </si>
+  <si>
+    <t>VICTOR'S AEGIS</t>
+  </si>
+  <si>
+    <t>On WIN, damage taken -30% for the next 2 rounds (including the win round)</t>
+  </si>
+  <si>
+    <t>WIN: รับดาเมจ-30% ต่อเนื่อง 2 รอบ</t>
+  </si>
+  <si>
+    <t>IRON CROWN</t>
+  </si>
+  <si>
+    <t>On WIN, also halve damage taken next round</t>
+  </si>
+  <si>
+    <t>WIN: ลดดาเมจครึ่งหนึ่งรอบถัดไปด้วย</t>
+  </si>
+  <si>
+    <t>SPECTRAL WALL</t>
+  </si>
+  <si>
+    <t>When you reflect damage, 20% chance to also dodge next round</t>
+  </si>
+  <si>
+    <t>สะท้อนดาเมจ 20% โอกาสหลบเทิร์นถัดไป</t>
+  </si>
+  <si>
+    <t>REFLECT STEP</t>
+  </si>
+  <si>
+    <t>When you reflect damage, heal 20% of the reflected amount</t>
+  </si>
+  <si>
+    <t>สะท้อนดาเมจ ฟื้น HP 20% ของดาเมจที่สะท้อนได้</t>
+  </si>
+  <si>
+    <t>IRON SKY</t>
+  </si>
+  <si>
+    <t>Both on WIN and LOSE, reduce damage taken by an extra 15%</t>
+  </si>
+  <si>
+    <t>WIN/LOSE ลดดาเมจเพิ่ม 15% ทั้ง 2 กรณี</t>
+  </si>
+  <si>
+    <t>ETERNAL WALL</t>
+  </si>
+  <si>
+    <t>The reflect and damage-halving effects can both trigger in the same turn</t>
+  </si>
+  <si>
+    <t>สะท้อนและลดดาเมจ (halve) เกิดพร้อมกันได้ในเทิร์นเดียว</t>
+  </si>
+  <si>
+    <t>DOUBLE EVASION</t>
+  </si>
+  <si>
+    <t>On a successful dodge, 20% chance to dodge again next round</t>
+  </si>
+  <si>
+    <t>หลบสำเร็จ 20% โอกาสหลบซ้ำเทิร์นถัดไป</t>
+  </si>
+  <si>
+    <t>GHOST WING</t>
+  </si>
+  <si>
+    <t>On a successful dodge, damage taken -30% for the next 2 turns</t>
+  </si>
+  <si>
+    <t>หลบสำเร็จ รับดาเมจ-30% อีก 2 เทิร์น</t>
+  </si>
+  <si>
+    <t>PHANTOM WALL</t>
+  </si>
+  <si>
+    <t>On a successful dodge, guarantee the damage-halving effect next round</t>
+  </si>
+  <si>
+    <t>หลบสำเร็จ เทิร์นถัดไปลดดาเมจครึ่งหนึ่งการันตี</t>
+  </si>
+  <si>
+    <t>SKY STEP</t>
+  </si>
+  <si>
+    <t>On a successful dodge, heal an extra 10% HP (total 25%)</t>
+  </si>
+  <si>
+    <t>⚖️</t>
+  </si>
+  <si>
+    <t>AEGIS STEP</t>
+  </si>
+  <si>
+    <t>10% chance to halve damage taken while also healing 10% HP that turn</t>
+  </si>
+  <si>
+    <t>10% โอกาสลดดาเมจครึ่งหนึ่ง พร้อมฟื้น HP 10%</t>
+  </si>
+  <si>
+    <t>FORTRESS WING</t>
+  </si>
+  <si>
+    <t>On WIN, guarantee the damage-halving effect</t>
+  </si>
+  <si>
+    <t>WIN: ลดดาเมจครึ่งหนึ่งการันตี</t>
+  </si>
+  <si>
+    <t>SYMBEAST — Fusion Passives v2 (proposal, ยังไม่ implement) — Approach B: 1 new half-strength Echo passive per Evolve II form (40 total, not per-pair)</t>
+  </si>
+  <si>
+    <t>Fusion = choose/random 1 of the 2 parents' own Evolve II form -&gt; egg inherits that form's Echo passive (numbers ~halved, freshly coded, no shared battle-state vars, so it never conflicts with any natural passive)</t>
+  </si>
+  <si>
+    <t>Evolve II Form | Icon | Echo Passive Name | Effect (EN) | Effect (TH)</t>
+  </si>
+  <si>
+    <t>Evolve II Form</t>
+  </si>
+  <si>
+    <t>Echo Passive Name</t>
+  </si>
+  <si>
+    <t>RAGING ECHO</t>
+  </si>
+  <si>
+    <t>On WIN: damage dealt +8% per stack (max 5 stacks per battle)</t>
+  </si>
+  <si>
+    <t>เมื่อ WIN ดาเมจเพิ่มขึ้นครั้งละ 8% (สะสมสูงสุด 5 ครั้ง)</t>
+  </si>
+  <si>
+    <t>🗡</t>
+  </si>
+  <si>
+    <t>WINDBLADE ECHO</t>
+  </si>
+  <si>
+    <t>☯️</t>
+  </si>
+  <si>
+    <t>CRIMSON ECHO</t>
+  </si>
+  <si>
+    <t>Every round: ATK+5% and SPD+5% (max 3 stacks per battle)</t>
+  </si>
+  <si>
+    <t>ทุกรอบ ATK+5% และ SPD+5% (สะสมสูงสุด 3 ครั้ง)</t>
+  </si>
+  <si>
+    <t>🦖</t>
+  </si>
+  <si>
+    <t>KAIJU ECHO</t>
+  </si>
+  <si>
+    <t>On LOSE: next round ATK+25%, DEF+25%, and 12% chance to burn the enemy</t>
+  </si>
+  <si>
+    <t>เมื่อ LOSE รอบถัดไป ATK+25%, DEF+25% และ 12% โอกาสทำให้ศัตรูติดเผาไหม้</t>
+  </si>
+  <si>
+    <t>FIGHTER ECHO</t>
+  </si>
+  <si>
+    <t>On LOSE: damage dealt +35% that turn</t>
+  </si>
+  <si>
+    <t>เมื่อ LOSE ดาเมจเพิ่มขึ้น 35% ในเทิร์นนั้น</t>
+  </si>
+  <si>
+    <t>NINJA ECHO</t>
+  </si>
+  <si>
+    <t>12% chance to fully dodge; on dodge, crit chance +50% next attack</t>
+  </si>
+  <si>
+    <t>12% โอกาสหลบการโจมตี เมื่อหลบสำเร็จ โอกาสคริ+50% ในการโจมตีถัดไป</t>
+  </si>
+  <si>
+    <t>WARRIOR ECHO</t>
+  </si>
+  <si>
+    <t>🛡</t>
+  </si>
+  <si>
+    <t>ARMOR ECHO</t>
+  </si>
+  <si>
+    <t>TYRANT ECHO</t>
+  </si>
+  <si>
+    <t>Damage dealt +10% and lifesteal +5%</t>
+  </si>
+  <si>
+    <t>ดาเมจที่สร้างเพิ่มขึ้น 10% และดูดเลือดเพิ่ม 5%</t>
+  </si>
+  <si>
+    <t>AGILE ECHO</t>
+  </si>
+  <si>
+    <t>12% chance to attack twice</t>
+  </si>
+  <si>
+    <t>12% โอกาสโจมตี 2 ครั้ง</t>
+  </si>
+  <si>
+    <t>🔮</t>
+  </si>
+  <si>
+    <t>RUNE ECHO</t>
+  </si>
+  <si>
+    <t>FULLARMOR ECHO</t>
+  </si>
+  <si>
+    <t>STRONG ECHO</t>
+  </si>
+  <si>
+    <t>On WIN: damage dealt +10% and 8% chance to stun the enemy for 1 round</t>
+  </si>
+  <si>
+    <t>เมื่อ WIN ดาเมจเพิ่มขึ้น 10% และ 8% โอกาส Stun ศัตรู 1 รอบ</t>
+  </si>
+  <si>
+    <t>🌩</t>
+  </si>
+  <si>
+    <t>STORM ECHO</t>
+  </si>
+  <si>
+    <t>THUNDERCLOUD ECHO</t>
+  </si>
+  <si>
+    <t>BULWARK ECHO</t>
+  </si>
+  <si>
+    <t>WARLORD ECHO</t>
+  </si>
+  <si>
+    <t>Damage dealt +10%; 5% chance to attack 4 times</t>
+  </si>
+  <si>
+    <t>ดาเมจที่สร้างเพิ่มขึ้น 10% และมีโอกาส 5% ที่จะโจมตี 4 ครั้ง</t>
+  </si>
+  <si>
+    <t>KING ECHO</t>
+  </si>
+  <si>
+    <t>10% chance to fully dodge; on dodge, ATK/DEF/SPD +5% (max 5 stacks per battle)</t>
+  </si>
+  <si>
+    <t>10% โอกาสหลบการโจมตี เมื่อหลบสำเร็จ ATK/DEF/SPD+5% (สะสมสูงสุด 5 ครั้ง)</t>
+  </si>
+  <si>
+    <t>SOUL ECHO</t>
+  </si>
+  <si>
+    <t>On WIN: ATK+12% and 12% chance to burn the enemy; on LOSE: dodge +12% and damage dealt +12% that round</t>
+  </si>
+  <si>
+    <t>เมื่อ WIN: ATK+12% และ 12% โอกาสทำให้ศัตรูติดเผาไหม้ เมื่อ LOSE: โอกาสหลบ+12% และดาเมจเพิ่ม 12% ในรอบนั้น</t>
+  </si>
+  <si>
+    <t>ROLLING ECHO</t>
+  </si>
+  <si>
+    <t>Damage taken -10%; every 3 rounds the attack deals +25% damage and cannot miss</t>
+  </si>
+  <si>
+    <t>ลดดาเมจที่รับ 10% และทุกๆ 3 รอบจะโจมตีแรงขึ้น 25% และไม่พลาดเป้า</t>
+  </si>
+  <si>
+    <t>BLAZING ECHO</t>
+  </si>
+  <si>
+    <t>On WIN: damage dealt +8% and DEF +8% per stack (max 3 stacks), 10% chance to poison the enemy</t>
+  </si>
+  <si>
+    <t>เมื่อ WIN ดาเมจ+8% และ DEF+8% สะสม (สูงสุด 3 ครั้ง) และ 10% โอกาสทำให้ศัตรูติดพิษ</t>
+  </si>
+  <si>
+    <t>SWIFT ECHO</t>
+  </si>
+  <si>
+    <t>Every 3 turns: reflects 35% of damage taken, recovers 5% HP, and 25% chance to poison the enemy</t>
+  </si>
+  <si>
+    <t>ทุก 3 เทิร์น สะท้อนดาเมจที่รับ 35% ฟื้นฟู HP 5% และ 25% โอกาสทำให้ศัตรูติดพิษ</t>
+  </si>
+  <si>
+    <t>POISON ECHO</t>
+  </si>
+  <si>
+    <t>Damage taken -5%; 12% chance to poison the enemy when hit (6% MaxHP/turn, 3 turns)</t>
+  </si>
+  <si>
+    <t>ลดดาเมจที่รับ 5% และ 12% โอกาสทำให้ศัตรูติดพิษเมื่อถูกโจมตี (6% MaxHP/เทิร์น นาน 3 เทิร์น)</t>
+  </si>
+  <si>
+    <t>🏰</t>
+  </si>
+  <si>
+    <t>GUARDIAN ECHO</t>
+  </si>
+  <si>
+    <t>Damage taken -12%; while HP &lt; 50%, reflects an extra 12% of damage taken back</t>
+  </si>
+  <si>
+    <t>ลดดาเมจที่รับ 12% และเมื่อ HP &lt; 50% จะสะท้อนดาเมจเพิ่มอีก 12%</t>
+  </si>
+  <si>
+    <t>🌑</t>
+  </si>
+  <si>
+    <t>DARK ECHO</t>
+  </si>
+  <si>
+    <t>Damage dealt +10%, crit chance +12%, lifesteal 7%</t>
+  </si>
+  <si>
+    <t>ดาเมจที่สร้างเพิ่มขึ้น 10%, คริ+12%, ดูดเลือด 7%</t>
+  </si>
+  <si>
+    <t>SPECTER ECHO</t>
+  </si>
+  <si>
+    <t>10% chance to fully dodge; on dodge, the next attack hits twice</t>
+  </si>
+  <si>
+    <t>10% โอกาสหลบการโจมตี เมื่อหลบสำเร็จ การโจมตีถัดไปโจมตี 2 ครั้ง</t>
+  </si>
+  <si>
+    <t>🧙</t>
+  </si>
+  <si>
+    <t>MAGE ECHO</t>
+  </si>
+  <si>
+    <t>⚰️</t>
+  </si>
+  <si>
+    <t>GRAVE ECHO</t>
+  </si>
+  <si>
+    <t>🥋</t>
+  </si>
+  <si>
+    <t>FIGHT ECHO</t>
+  </si>
+  <si>
+    <t>On WIN: damage dealt +8%, dodge +3%, crit chance +3% per stack (max 3 stacks)</t>
+  </si>
+  <si>
+    <t>เมื่อ WIN ดาเมจ+8%, หลบ+3%, คริ+3% (สะสมสูงสุด 3 ครั้ง)</t>
+  </si>
+  <si>
+    <t>QUICK ECHO</t>
+  </si>
+  <si>
+    <t>12% chance to fully dodge; on dodge, the next attack pierces DEF and cannot miss</t>
+  </si>
+  <si>
+    <t>12% โอกาสหลบการโจมตี เมื่อหลบสำเร็จ การโจมตีถัดไปทะลุ DEF และไม่พลาดเป้า</t>
+  </si>
+  <si>
+    <t>PHOENIX ECHO</t>
+  </si>
+  <si>
+    <t>Every attack has an 8% chance to burn the enemy; once per battle when HP &lt; 30%: heal 50% HP + ATK/DEF/SPD +8%</t>
+  </si>
+  <si>
+    <t>ทุกการโจมตีมีโอกาส 8% ทำให้ศัตรูติดเผาไหม้ เมื่อ HP&lt;30% (ครั้งเดียว): ฟื้น HP 50% + ATK/DEF/SPD +8%</t>
+  </si>
+  <si>
+    <t>IRON ECHO</t>
+  </si>
+  <si>
+    <t>On LOSE: damage taken -8% per stack (max 3 stacks per battle)</t>
+  </si>
+  <si>
+    <t>เมื่อ LOSE ลดดาเมจที่รับ 8% สะสม (สูงสุด 3 ครั้ง)</t>
+  </si>
+  <si>
+    <t>🔨</t>
+  </si>
+  <si>
+    <t>HAMMER ECHO</t>
+  </si>
+  <si>
+    <t>On WIN: damage dealt +10%, 8% chance to stun, and the attack pierces DEF</t>
+  </si>
+  <si>
+    <t>เมื่อ WIN ดาเมจ+10%, 8% โอกาสสตัน และโจมตีทะลุ DEF</t>
+  </si>
+  <si>
+    <t>❄️</t>
+  </si>
+  <si>
+    <t>CHILL ECHO</t>
+  </si>
+  <si>
+    <t>Every 3 turns: dodges 50% and attacks through DEF with ATK +25%</t>
+  </si>
+  <si>
+    <t>ทุก 3 เทิร์น: หลบ 50% และโจมตีทะลุ DEF ด้วย ATK+25%</t>
+  </si>
+  <si>
+    <t>🌿</t>
+  </si>
+  <si>
+    <t>GAIA ECHO</t>
+  </si>
+  <si>
+    <t>Every 3 rounds: recovers 8% of Max HP and ATK/DEF +10% that round</t>
+  </si>
+  <si>
+    <t>ทุก 3 รอบ: ฟื้น HP 8% ของ Max HP และ ATK/DEF+10% ในรอบนั้น</t>
+  </si>
+  <si>
+    <t>FATTY ECHO</t>
+  </si>
+  <si>
+    <t>Damage taken -10%; while HP &gt; 70%, ATK/DEF +15%; while HP &lt; 70%, ATK +25%</t>
+  </si>
+  <si>
+    <t>ลดดาเมจที่รับ 10% เมื่อ HP &gt; 70% ATK/DEF+15% เมื่อ HP &lt; 70% ATK+25%</t>
+  </si>
+  <si>
+    <t>GUANLET ECHO</t>
+  </si>
+  <si>
+    <t>On LOSE: damage dealt +8% per stack (max 5 stacks per battle)</t>
+  </si>
+  <si>
+    <t>เมื่อ LOSE ดาเมจเพิ่มขึ้นครั้งละ 8% (สะสมสูงสุด 5 ครั้ง)</t>
+  </si>
+  <si>
+    <t>BASTION ECHO</t>
+  </si>
+  <si>
+    <t>10% chance to fully dodge; every 3 turns, attacks cannot miss, deal +25% damage, and guarantee a crit</t>
+  </si>
+  <si>
+    <t>10% โอกาสหลบการโจมตี ทุก 3 เทิร์น โจมตีไม่พลาดเป้า ดาเมจ+25% และติดคริแน่นอน</t>
+  </si>
+  <si>
+    <t>💎</t>
+  </si>
+  <si>
+    <t>CRYSTAL ECHO</t>
+  </si>
+  <si>
+    <t>GOLEM ECHO</t>
+  </si>
+  <si>
+    <t>Damage taken -10%; while HP &lt; 30%, ATK +15% and recovers 2.5% HP each round</t>
+  </si>
+  <si>
+    <t>ลดดาเมจที่รับ 10% เมื่อ HP &lt; 30% ATK+15% และฟื้นฟู HP 2.5%</t>
+  </si>
+  <si>
+    <t>12% โอกาสหลบการโจมตี เมื่อหลบสำเร็จโต้กลับดาเมจ 75%</t>
+  </si>
+  <si>
+    <t>12% chance to fully dodge; on dodge, counter-attacks for 75% damage</t>
+  </si>
+  <si>
+    <t>12% โอกาสรับดาเมจครึ่งหนึ่งและโต้กลับด้วยดาเมจ 75%</t>
+  </si>
+  <si>
+    <t>12% chance to take half damage and counter-attack for 75% damage</t>
+  </si>
+  <si>
+    <t>Damage taken -10%; 25% chance to counter-attack for 75% damage</t>
+  </si>
+  <si>
+    <t>ลดดาเมจที่รับ 10% และ 25% โอกาสโต้กลับด้วยดาเมจ 75%</t>
+  </si>
+  <si>
+    <t>8% โอกาสสตันศัตรู และทุกรอบได้รับ Rune สุ่ม: ATK+50% หรือ DEF+50%</t>
+  </si>
+  <si>
+    <t>เมื่อ HP &lt; 50% ลดดาเมจที่รับ 10% และโต้กลับด้วยดาเมจ 75%</t>
+  </si>
+  <si>
+    <t>8% chance to stun the enemy; each round gains a random Rune: ATK+50% or DEF+50%</t>
+  </si>
+  <si>
+    <t>While HP &lt; 50%: damage taken -10% and counter-attacks for 75% damage</t>
+  </si>
+  <si>
+    <t>10% โอกาสหลบการโจมตี เมื่อหลบสำเร็จ ATK+50% รอบถัดไป</t>
+  </si>
+  <si>
+    <t>10% chance to fully dodge; on dodge, ATK +50% next round</t>
+  </si>
+  <si>
+    <t>8% โอกาส Stun ศัตรู ถ้าไม่ติดจะได้โอกาสหลบ 25% แทนในรอบนั้น</t>
+  </si>
+  <si>
+    <t>ลดดาเมจที่รับ 10% และเมื่อถูกโจมตีมีโอกาส 15% ทำให้อีกฝ่าย Stun 1 รอบ</t>
+  </si>
+  <si>
+    <t>8% chance to stun the enemy; if not stunned, gains 25% dodge that round instead</t>
+  </si>
+  <si>
+    <t>Damage taken -10%; when hit, 15% chance to stun the attacker for 1 round</t>
+  </si>
+  <si>
+    <t>ลดดาเมจที่รับ 12% และมีโอกาส 25% ฟื้นฟู HP 5%</t>
+  </si>
+  <si>
+    <t>Damage taken -12%; 25% chance to recover 5% HP each round</t>
+  </si>
+  <si>
+    <t>เมื่อ HP &gt; 50%: ATK+12% เมื่อ HP &lt; 50%: DEF+12%, โต้กลับดาเมจ 75%, 5% โอกาสสตันเมื่อโดนโจมตี</t>
+  </si>
+  <si>
+    <t>While HP &gt; 50%: ATK+12%. While HP &lt; 50%: DEF+12%, counter-attacks for 75% damage, 5% chance to stun when hit</t>
+  </si>
+  <si>
+    <t>On WIN: curses the enemy, ATK -12% for 2 turns; on DRAW: enemy cannot heal for 3 turns; on LOSE: damage taken -5%</t>
+  </si>
+  <si>
+    <t>เมื่อ WIN: สาปศัตรู ATK-12% นาน 2 เทิร์น เมื่อ DRAW: สาปให้ศัตรูฟื้นฟู HP ไม่ได้ 3 เทิร์น เมื่อ LOSE: ลดดาเมจที่รับ 5%</t>
   </si>
 </sst>
 </file>
@@ -13042,6 +14049,2048 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBF0D8DD-BA0A-4ACD-BB65-CCCC29CBF622}">
+  <dimension ref="A1:G59"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="3" width="12.69921875" customWidth="1"/>
+    <col min="4" max="4" width="6.69921875" customWidth="1"/>
+    <col min="5" max="5" width="20.69921875" customWidth="1"/>
+    <col min="6" max="7" width="55.69921875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>1656</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>1657</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>1658</v>
+      </c>
+      <c r="B4" t="s">
+        <v>1659</v>
+      </c>
+      <c r="C4" t="s">
+        <v>1660</v>
+      </c>
+      <c r="D4" t="s">
+        <v>3</v>
+      </c>
+      <c r="E4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F4" t="s">
+        <v>267</v>
+      </c>
+      <c r="G4" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>1661</v>
+      </c>
+      <c r="B5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" t="s">
+        <v>1662</v>
+      </c>
+      <c r="E5" t="s">
+        <v>1663</v>
+      </c>
+      <c r="F5" t="s">
+        <v>1664</v>
+      </c>
+      <c r="G5" t="s">
+        <v>1665</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>1661</v>
+      </c>
+      <c r="B6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6" t="s">
+        <v>1666</v>
+      </c>
+      <c r="E6" t="s">
+        <v>1667</v>
+      </c>
+      <c r="F6" t="s">
+        <v>1668</v>
+      </c>
+      <c r="G6" t="s">
+        <v>1669</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>1661</v>
+      </c>
+      <c r="B7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" t="s">
+        <v>1670</v>
+      </c>
+      <c r="E7" t="s">
+        <v>1671</v>
+      </c>
+      <c r="F7" t="s">
+        <v>1672</v>
+      </c>
+      <c r="G7" t="s">
+        <v>1673</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>1661</v>
+      </c>
+      <c r="B8" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" t="s">
+        <v>23</v>
+      </c>
+      <c r="D8" t="s">
+        <v>15</v>
+      </c>
+      <c r="E8" t="s">
+        <v>1674</v>
+      </c>
+      <c r="F8" t="s">
+        <v>1675</v>
+      </c>
+      <c r="G8" t="s">
+        <v>1676</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>1661</v>
+      </c>
+      <c r="B9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" t="s">
+        <v>27</v>
+      </c>
+      <c r="D9" t="s">
+        <v>1677</v>
+      </c>
+      <c r="E9" t="s">
+        <v>1678</v>
+      </c>
+      <c r="F9" t="s">
+        <v>1679</v>
+      </c>
+      <c r="G9" t="s">
+        <v>1680</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>1661</v>
+      </c>
+      <c r="B10" t="s">
+        <v>31</v>
+      </c>
+      <c r="C10" t="s">
+        <v>31</v>
+      </c>
+      <c r="D10" t="s">
+        <v>1681</v>
+      </c>
+      <c r="E10" t="s">
+        <v>1682</v>
+      </c>
+      <c r="F10" t="s">
+        <v>1683</v>
+      </c>
+      <c r="G10" t="s">
+        <v>1684</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>1661</v>
+      </c>
+      <c r="B11" t="s">
+        <v>35</v>
+      </c>
+      <c r="C11" t="s">
+        <v>35</v>
+      </c>
+      <c r="D11" t="s">
+        <v>1685</v>
+      </c>
+      <c r="E11" t="s">
+        <v>1686</v>
+      </c>
+      <c r="F11" t="s">
+        <v>1687</v>
+      </c>
+      <c r="G11" t="s">
+        <v>1688</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>1661</v>
+      </c>
+      <c r="B12" t="s">
+        <v>39</v>
+      </c>
+      <c r="C12" t="s">
+        <v>39</v>
+      </c>
+      <c r="D12" t="s">
+        <v>1689</v>
+      </c>
+      <c r="E12" t="s">
+        <v>1690</v>
+      </c>
+      <c r="F12" t="s">
+        <v>1691</v>
+      </c>
+      <c r="G12" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>1661</v>
+      </c>
+      <c r="B13" t="s">
+        <v>43</v>
+      </c>
+      <c r="C13" t="s">
+        <v>43</v>
+      </c>
+      <c r="D13" t="s">
+        <v>1693</v>
+      </c>
+      <c r="E13" t="s">
+        <v>1694</v>
+      </c>
+      <c r="F13" t="s">
+        <v>1695</v>
+      </c>
+      <c r="G13" t="s">
+        <v>1696</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>1661</v>
+      </c>
+      <c r="B14" t="s">
+        <v>47</v>
+      </c>
+      <c r="C14" t="s">
+        <v>47</v>
+      </c>
+      <c r="D14" t="s">
+        <v>46</v>
+      </c>
+      <c r="E14" t="s">
+        <v>1697</v>
+      </c>
+      <c r="F14" t="s">
+        <v>1698</v>
+      </c>
+      <c r="G14" t="s">
+        <v>1699</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>1700</v>
+      </c>
+      <c r="B15" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15" t="s">
+        <v>16</v>
+      </c>
+      <c r="D15" t="s">
+        <v>1701</v>
+      </c>
+      <c r="E15" t="s">
+        <v>1702</v>
+      </c>
+      <c r="F15" t="s">
+        <v>1703</v>
+      </c>
+      <c r="G15" t="s">
+        <v>1704</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>1700</v>
+      </c>
+      <c r="B16" t="s">
+        <v>12</v>
+      </c>
+      <c r="C16" t="s">
+        <v>20</v>
+      </c>
+      <c r="D16" t="s">
+        <v>1705</v>
+      </c>
+      <c r="E16" t="s">
+        <v>1706</v>
+      </c>
+      <c r="F16" t="s">
+        <v>1707</v>
+      </c>
+      <c r="G16" t="s">
+        <v>1708</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>1700</v>
+      </c>
+      <c r="B17" t="s">
+        <v>12</v>
+      </c>
+      <c r="C17" t="s">
+        <v>23</v>
+      </c>
+      <c r="D17" t="s">
+        <v>15</v>
+      </c>
+      <c r="E17" t="s">
+        <v>1709</v>
+      </c>
+      <c r="F17" t="s">
+        <v>1710</v>
+      </c>
+      <c r="G17" t="s">
+        <v>1711</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>1700</v>
+      </c>
+      <c r="B18" t="s">
+        <v>12</v>
+      </c>
+      <c r="C18" t="s">
+        <v>27</v>
+      </c>
+      <c r="D18" t="s">
+        <v>1712</v>
+      </c>
+      <c r="E18" t="s">
+        <v>1713</v>
+      </c>
+      <c r="F18" t="s">
+        <v>1714</v>
+      </c>
+      <c r="G18" t="s">
+        <v>1715</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>1700</v>
+      </c>
+      <c r="B19" t="s">
+        <v>12</v>
+      </c>
+      <c r="C19" t="s">
+        <v>31</v>
+      </c>
+      <c r="D19" t="s">
+        <v>498</v>
+      </c>
+      <c r="E19" t="s">
+        <v>1716</v>
+      </c>
+      <c r="F19" t="s">
+        <v>1717</v>
+      </c>
+      <c r="G19" t="s">
+        <v>1718</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>1700</v>
+      </c>
+      <c r="B20" t="s">
+        <v>12</v>
+      </c>
+      <c r="C20" t="s">
+        <v>35</v>
+      </c>
+      <c r="D20" t="s">
+        <v>1719</v>
+      </c>
+      <c r="E20" t="s">
+        <v>1720</v>
+      </c>
+      <c r="F20" t="s">
+        <v>1721</v>
+      </c>
+      <c r="G20" t="s">
+        <v>1722</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>1700</v>
+      </c>
+      <c r="B21" t="s">
+        <v>12</v>
+      </c>
+      <c r="C21" t="s">
+        <v>39</v>
+      </c>
+      <c r="D21" t="s">
+        <v>1723</v>
+      </c>
+      <c r="E21" t="s">
+        <v>1724</v>
+      </c>
+      <c r="F21" t="s">
+        <v>1725</v>
+      </c>
+      <c r="G21" t="s">
+        <v>1726</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>1700</v>
+      </c>
+      <c r="B22" t="s">
+        <v>12</v>
+      </c>
+      <c r="C22" t="s">
+        <v>43</v>
+      </c>
+      <c r="D22" t="s">
+        <v>498</v>
+      </c>
+      <c r="E22" t="s">
+        <v>1727</v>
+      </c>
+      <c r="F22" t="s">
+        <v>1728</v>
+      </c>
+      <c r="G22" t="s">
+        <v>1729</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>1700</v>
+      </c>
+      <c r="B23" t="s">
+        <v>12</v>
+      </c>
+      <c r="C23" t="s">
+        <v>47</v>
+      </c>
+      <c r="D23" t="s">
+        <v>1730</v>
+      </c>
+      <c r="E23" t="s">
+        <v>1731</v>
+      </c>
+      <c r="F23" t="s">
+        <v>1732</v>
+      </c>
+      <c r="G23" t="s">
+        <v>1733</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>1700</v>
+      </c>
+      <c r="B24" t="s">
+        <v>16</v>
+      </c>
+      <c r="C24" t="s">
+        <v>20</v>
+      </c>
+      <c r="D24" t="s">
+        <v>1670</v>
+      </c>
+      <c r="E24" t="s">
+        <v>1734</v>
+      </c>
+      <c r="F24" t="s">
+        <v>1735</v>
+      </c>
+      <c r="G24" t="s">
+        <v>1736</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>1700</v>
+      </c>
+      <c r="B25" t="s">
+        <v>16</v>
+      </c>
+      <c r="C25" t="s">
+        <v>23</v>
+      </c>
+      <c r="D25" t="s">
+        <v>15</v>
+      </c>
+      <c r="E25" t="s">
+        <v>1737</v>
+      </c>
+      <c r="F25" t="s">
+        <v>1738</v>
+      </c>
+      <c r="G25" t="s">
+        <v>1739</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>1700</v>
+      </c>
+      <c r="B26" t="s">
+        <v>16</v>
+      </c>
+      <c r="C26" t="s">
+        <v>27</v>
+      </c>
+      <c r="D26" t="s">
+        <v>1740</v>
+      </c>
+      <c r="E26" t="s">
+        <v>1741</v>
+      </c>
+      <c r="F26" t="s">
+        <v>1742</v>
+      </c>
+      <c r="G26" t="s">
+        <v>1743</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>1700</v>
+      </c>
+      <c r="B27" t="s">
+        <v>16</v>
+      </c>
+      <c r="C27" t="s">
+        <v>31</v>
+      </c>
+      <c r="D27" t="s">
+        <v>1744</v>
+      </c>
+      <c r="E27" t="s">
+        <v>1745</v>
+      </c>
+      <c r="F27" t="s">
+        <v>1746</v>
+      </c>
+      <c r="G27" t="s">
+        <v>1747</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>1700</v>
+      </c>
+      <c r="B28" t="s">
+        <v>16</v>
+      </c>
+      <c r="C28" t="s">
+        <v>35</v>
+      </c>
+      <c r="D28" t="s">
+        <v>1748</v>
+      </c>
+      <c r="E28" t="s">
+        <v>1749</v>
+      </c>
+      <c r="F28" t="s">
+        <v>1750</v>
+      </c>
+      <c r="G28" t="s">
+        <v>1751</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>1700</v>
+      </c>
+      <c r="B29" t="s">
+        <v>16</v>
+      </c>
+      <c r="C29" t="s">
+        <v>39</v>
+      </c>
+      <c r="D29" t="s">
+        <v>1752</v>
+      </c>
+      <c r="E29" t="s">
+        <v>1753</v>
+      </c>
+      <c r="F29" t="s">
+        <v>1754</v>
+      </c>
+      <c r="G29" t="s">
+        <v>1755</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>1700</v>
+      </c>
+      <c r="B30" t="s">
+        <v>16</v>
+      </c>
+      <c r="C30" t="s">
+        <v>43</v>
+      </c>
+      <c r="D30" t="s">
+        <v>1693</v>
+      </c>
+      <c r="E30" t="s">
+        <v>1756</v>
+      </c>
+      <c r="F30" t="s">
+        <v>1757</v>
+      </c>
+      <c r="G30" t="s">
+        <v>1758</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>1700</v>
+      </c>
+      <c r="B31" t="s">
+        <v>16</v>
+      </c>
+      <c r="C31" t="s">
+        <v>47</v>
+      </c>
+      <c r="D31" t="s">
+        <v>498</v>
+      </c>
+      <c r="E31" t="s">
+        <v>1759</v>
+      </c>
+      <c r="F31" t="s">
+        <v>1760</v>
+      </c>
+      <c r="G31" t="s">
+        <v>1761</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>1700</v>
+      </c>
+      <c r="B32" t="s">
+        <v>20</v>
+      </c>
+      <c r="C32" t="s">
+        <v>23</v>
+      </c>
+      <c r="D32" t="s">
+        <v>1762</v>
+      </c>
+      <c r="E32" t="s">
+        <v>1763</v>
+      </c>
+      <c r="F32" t="s">
+        <v>1764</v>
+      </c>
+      <c r="G32" t="s">
+        <v>1765</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>1700</v>
+      </c>
+      <c r="B33" t="s">
+        <v>20</v>
+      </c>
+      <c r="C33" t="s">
+        <v>27</v>
+      </c>
+      <c r="D33" t="s">
+        <v>1670</v>
+      </c>
+      <c r="E33" t="s">
+        <v>1766</v>
+      </c>
+      <c r="F33" t="s">
+        <v>1767</v>
+      </c>
+      <c r="G33" t="s">
+        <v>1768</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>1700</v>
+      </c>
+      <c r="B34" t="s">
+        <v>20</v>
+      </c>
+      <c r="C34" t="s">
+        <v>31</v>
+      </c>
+      <c r="D34" t="s">
+        <v>1769</v>
+      </c>
+      <c r="E34" t="s">
+        <v>1770</v>
+      </c>
+      <c r="F34" t="s">
+        <v>1771</v>
+      </c>
+      <c r="G34" t="s">
+        <v>1772</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>1700</v>
+      </c>
+      <c r="B35" t="s">
+        <v>20</v>
+      </c>
+      <c r="C35" t="s">
+        <v>35</v>
+      </c>
+      <c r="D35" t="s">
+        <v>1773</v>
+      </c>
+      <c r="E35" t="s">
+        <v>1774</v>
+      </c>
+      <c r="F35" t="s">
+        <v>1775</v>
+      </c>
+      <c r="G35" t="s">
+        <v>1776</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>1700</v>
+      </c>
+      <c r="B36" t="s">
+        <v>20</v>
+      </c>
+      <c r="C36" t="s">
+        <v>39</v>
+      </c>
+      <c r="D36" t="s">
+        <v>1752</v>
+      </c>
+      <c r="E36" t="s">
+        <v>1777</v>
+      </c>
+      <c r="F36" t="s">
+        <v>1778</v>
+      </c>
+      <c r="G36" t="s">
+        <v>1779</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>1700</v>
+      </c>
+      <c r="B37" t="s">
+        <v>20</v>
+      </c>
+      <c r="C37" t="s">
+        <v>43</v>
+      </c>
+      <c r="D37" t="s">
+        <v>1693</v>
+      </c>
+      <c r="E37" t="s">
+        <v>1780</v>
+      </c>
+      <c r="F37" t="s">
+        <v>1781</v>
+      </c>
+      <c r="G37" t="s">
+        <v>1782</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>1700</v>
+      </c>
+      <c r="B38" t="s">
+        <v>20</v>
+      </c>
+      <c r="C38" t="s">
+        <v>47</v>
+      </c>
+      <c r="D38" t="s">
+        <v>1681</v>
+      </c>
+      <c r="E38" t="s">
+        <v>1783</v>
+      </c>
+      <c r="F38" t="s">
+        <v>1784</v>
+      </c>
+      <c r="G38" t="s">
+        <v>1785</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>1700</v>
+      </c>
+      <c r="B39" t="s">
+        <v>23</v>
+      </c>
+      <c r="C39" t="s">
+        <v>27</v>
+      </c>
+      <c r="D39" t="s">
+        <v>15</v>
+      </c>
+      <c r="E39" t="s">
+        <v>1786</v>
+      </c>
+      <c r="F39" t="s">
+        <v>1787</v>
+      </c>
+      <c r="G39" t="s">
+        <v>1788</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>1700</v>
+      </c>
+      <c r="B40" t="s">
+        <v>23</v>
+      </c>
+      <c r="C40" t="s">
+        <v>31</v>
+      </c>
+      <c r="D40" t="s">
+        <v>1769</v>
+      </c>
+      <c r="E40" t="s">
+        <v>1789</v>
+      </c>
+      <c r="F40" t="s">
+        <v>1790</v>
+      </c>
+      <c r="G40" t="s">
+        <v>1791</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>1700</v>
+      </c>
+      <c r="B41" t="s">
+        <v>23</v>
+      </c>
+      <c r="C41" t="s">
+        <v>35</v>
+      </c>
+      <c r="D41" t="s">
+        <v>1685</v>
+      </c>
+      <c r="E41" t="s">
+        <v>1792</v>
+      </c>
+      <c r="F41" t="s">
+        <v>1793</v>
+      </c>
+      <c r="G41" t="s">
+        <v>1794</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>1700</v>
+      </c>
+      <c r="B42" t="s">
+        <v>23</v>
+      </c>
+      <c r="C42" t="s">
+        <v>39</v>
+      </c>
+      <c r="D42" t="s">
+        <v>504</v>
+      </c>
+      <c r="E42" t="s">
+        <v>1795</v>
+      </c>
+      <c r="F42" t="s">
+        <v>1796</v>
+      </c>
+      <c r="G42" t="s">
+        <v>1797</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>1700</v>
+      </c>
+      <c r="B43" t="s">
+        <v>23</v>
+      </c>
+      <c r="C43" t="s">
+        <v>43</v>
+      </c>
+      <c r="D43" t="s">
+        <v>1239</v>
+      </c>
+      <c r="E43" t="s">
+        <v>1798</v>
+      </c>
+      <c r="F43" t="s">
+        <v>1799</v>
+      </c>
+      <c r="G43" t="s">
+        <v>1800</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>1700</v>
+      </c>
+      <c r="B44" t="s">
+        <v>23</v>
+      </c>
+      <c r="C44" t="s">
+        <v>47</v>
+      </c>
+      <c r="D44" t="s">
+        <v>1730</v>
+      </c>
+      <c r="E44" t="s">
+        <v>1801</v>
+      </c>
+      <c r="F44" t="s">
+        <v>1802</v>
+      </c>
+      <c r="G44" t="s">
+        <v>1803</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>1700</v>
+      </c>
+      <c r="B45" t="s">
+        <v>27</v>
+      </c>
+      <c r="C45" t="s">
+        <v>31</v>
+      </c>
+      <c r="D45" t="s">
+        <v>1677</v>
+      </c>
+      <c r="E45" t="s">
+        <v>1804</v>
+      </c>
+      <c r="F45" t="s">
+        <v>1805</v>
+      </c>
+      <c r="G45" t="s">
+        <v>1806</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>1700</v>
+      </c>
+      <c r="B46" t="s">
+        <v>27</v>
+      </c>
+      <c r="C46" t="s">
+        <v>35</v>
+      </c>
+      <c r="D46" t="s">
+        <v>1807</v>
+      </c>
+      <c r="E46" t="s">
+        <v>1808</v>
+      </c>
+      <c r="F46" t="s">
+        <v>1809</v>
+      </c>
+      <c r="G46" t="s">
+        <v>1810</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>1700</v>
+      </c>
+      <c r="B47" t="s">
+        <v>27</v>
+      </c>
+      <c r="C47" t="s">
+        <v>39</v>
+      </c>
+      <c r="D47" t="s">
+        <v>1811</v>
+      </c>
+      <c r="E47" t="s">
+        <v>1812</v>
+      </c>
+      <c r="F47" t="s">
+        <v>1813</v>
+      </c>
+      <c r="G47" t="s">
+        <v>1814</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>1700</v>
+      </c>
+      <c r="B48" t="s">
+        <v>27</v>
+      </c>
+      <c r="C48" t="s">
+        <v>43</v>
+      </c>
+      <c r="D48" t="s">
+        <v>1807</v>
+      </c>
+      <c r="E48" t="s">
+        <v>1815</v>
+      </c>
+      <c r="F48" t="s">
+        <v>1816</v>
+      </c>
+      <c r="G48" t="s">
+        <v>1817</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>1700</v>
+      </c>
+      <c r="B49" t="s">
+        <v>27</v>
+      </c>
+      <c r="C49" t="s">
+        <v>47</v>
+      </c>
+      <c r="D49" t="s">
+        <v>1807</v>
+      </c>
+      <c r="E49" t="s">
+        <v>1818</v>
+      </c>
+      <c r="F49" t="s">
+        <v>1819</v>
+      </c>
+      <c r="G49" t="s">
+        <v>1820</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>1700</v>
+      </c>
+      <c r="B50" t="s">
+        <v>31</v>
+      </c>
+      <c r="C50" t="s">
+        <v>35</v>
+      </c>
+      <c r="D50" t="s">
+        <v>1685</v>
+      </c>
+      <c r="E50" t="s">
+        <v>1821</v>
+      </c>
+      <c r="F50" t="s">
+        <v>1822</v>
+      </c>
+      <c r="G50" t="s">
+        <v>1823</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>1700</v>
+      </c>
+      <c r="B51" t="s">
+        <v>31</v>
+      </c>
+      <c r="C51" t="s">
+        <v>39</v>
+      </c>
+      <c r="D51" t="s">
+        <v>1752</v>
+      </c>
+      <c r="E51" t="s">
+        <v>1824</v>
+      </c>
+      <c r="F51" t="s">
+        <v>1825</v>
+      </c>
+      <c r="G51" t="s">
+        <v>1826</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>1700</v>
+      </c>
+      <c r="B52" t="s">
+        <v>31</v>
+      </c>
+      <c r="C52" t="s">
+        <v>43</v>
+      </c>
+      <c r="D52" t="s">
+        <v>1693</v>
+      </c>
+      <c r="E52" t="s">
+        <v>1827</v>
+      </c>
+      <c r="F52" t="s">
+        <v>1828</v>
+      </c>
+      <c r="G52" t="s">
+        <v>1829</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>1700</v>
+      </c>
+      <c r="B53" t="s">
+        <v>31</v>
+      </c>
+      <c r="C53" t="s">
+        <v>47</v>
+      </c>
+      <c r="D53" t="s">
+        <v>46</v>
+      </c>
+      <c r="E53" t="s">
+        <v>1830</v>
+      </c>
+      <c r="F53" t="s">
+        <v>1831</v>
+      </c>
+      <c r="G53" t="s">
+        <v>1832</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>1700</v>
+      </c>
+      <c r="B54" t="s">
+        <v>35</v>
+      </c>
+      <c r="C54" t="s">
+        <v>39</v>
+      </c>
+      <c r="D54" t="s">
+        <v>1752</v>
+      </c>
+      <c r="E54" t="s">
+        <v>1833</v>
+      </c>
+      <c r="F54" t="s">
+        <v>1834</v>
+      </c>
+      <c r="G54" t="s">
+        <v>1835</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>1700</v>
+      </c>
+      <c r="B55" t="s">
+        <v>35</v>
+      </c>
+      <c r="C55" t="s">
+        <v>43</v>
+      </c>
+      <c r="D55" t="s">
+        <v>1693</v>
+      </c>
+      <c r="E55" t="s">
+        <v>1836</v>
+      </c>
+      <c r="F55" t="s">
+        <v>1837</v>
+      </c>
+      <c r="G55" t="s">
+        <v>1838</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>1700</v>
+      </c>
+      <c r="B56" t="s">
+        <v>35</v>
+      </c>
+      <c r="C56" t="s">
+        <v>47</v>
+      </c>
+      <c r="D56" t="s">
+        <v>46</v>
+      </c>
+      <c r="E56" t="s">
+        <v>1839</v>
+      </c>
+      <c r="F56" t="s">
+        <v>1840</v>
+      </c>
+      <c r="G56" t="s">
+        <v>1841</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
+        <v>1700</v>
+      </c>
+      <c r="B57" t="s">
+        <v>39</v>
+      </c>
+      <c r="C57" t="s">
+        <v>43</v>
+      </c>
+      <c r="D57" t="s">
+        <v>1693</v>
+      </c>
+      <c r="E57" t="s">
+        <v>1842</v>
+      </c>
+      <c r="F57" t="s">
+        <v>1843</v>
+      </c>
+      <c r="G57" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>1700</v>
+      </c>
+      <c r="B58" t="s">
+        <v>39</v>
+      </c>
+      <c r="C58" t="s">
+        <v>47</v>
+      </c>
+      <c r="D58" t="s">
+        <v>1844</v>
+      </c>
+      <c r="E58" t="s">
+        <v>1845</v>
+      </c>
+      <c r="F58" t="s">
+        <v>1846</v>
+      </c>
+      <c r="G58" t="s">
+        <v>1847</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>1700</v>
+      </c>
+      <c r="B59" t="s">
+        <v>43</v>
+      </c>
+      <c r="C59" t="s">
+        <v>47</v>
+      </c>
+      <c r="D59" t="s">
+        <v>46</v>
+      </c>
+      <c r="E59" t="s">
+        <v>1848</v>
+      </c>
+      <c r="F59" t="s">
+        <v>1849</v>
+      </c>
+      <c r="G59" t="s">
+        <v>1850</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F00FD1CF-924F-4FD0-B28B-32154B63F96A}">
+  <dimension ref="A1:E45"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="18.69921875" customWidth="1"/>
+    <col min="2" max="2" width="6.69921875" customWidth="1"/>
+    <col min="3" max="3" width="18.69921875" customWidth="1"/>
+    <col min="4" max="5" width="60.69921875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>1851</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>1852</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>1853</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>1854</v>
+      </c>
+      <c r="B5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5" t="s">
+        <v>1855</v>
+      </c>
+      <c r="D5" t="s">
+        <v>267</v>
+      </c>
+      <c r="E5" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>59</v>
+      </c>
+      <c r="B6" t="s">
+        <v>1662</v>
+      </c>
+      <c r="C6" t="s">
+        <v>1856</v>
+      </c>
+      <c r="D6" t="s">
+        <v>1857</v>
+      </c>
+      <c r="E6" t="s">
+        <v>1858</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>64</v>
+      </c>
+      <c r="B7" t="s">
+        <v>1859</v>
+      </c>
+      <c r="C7" t="s">
+        <v>1860</v>
+      </c>
+      <c r="D7" t="s">
+        <v>1970</v>
+      </c>
+      <c r="E7" t="s">
+        <v>1969</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>69</v>
+      </c>
+      <c r="B8" t="s">
+        <v>1861</v>
+      </c>
+      <c r="C8" t="s">
+        <v>1862</v>
+      </c>
+      <c r="D8" t="s">
+        <v>1863</v>
+      </c>
+      <c r="E8" t="s">
+        <v>1864</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>73</v>
+      </c>
+      <c r="B9" t="s">
+        <v>1865</v>
+      </c>
+      <c r="C9" t="s">
+        <v>1866</v>
+      </c>
+      <c r="D9" t="s">
+        <v>1867</v>
+      </c>
+      <c r="E9" t="s">
+        <v>1868</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>76</v>
+      </c>
+      <c r="B10" t="s">
+        <v>1712</v>
+      </c>
+      <c r="C10" t="s">
+        <v>1869</v>
+      </c>
+      <c r="D10" t="s">
+        <v>1870</v>
+      </c>
+      <c r="E10" t="s">
+        <v>1871</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>80</v>
+      </c>
+      <c r="B11" t="s">
+        <v>1748</v>
+      </c>
+      <c r="C11" t="s">
+        <v>1872</v>
+      </c>
+      <c r="D11" t="s">
+        <v>1873</v>
+      </c>
+      <c r="E11" t="s">
+        <v>1874</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>84</v>
+      </c>
+      <c r="B12" t="s">
+        <v>1666</v>
+      </c>
+      <c r="C12" t="s">
+        <v>1875</v>
+      </c>
+      <c r="D12" t="s">
+        <v>1972</v>
+      </c>
+      <c r="E12" t="s">
+        <v>1971</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>88</v>
+      </c>
+      <c r="B13" t="s">
+        <v>1876</v>
+      </c>
+      <c r="C13" t="s">
+        <v>1877</v>
+      </c>
+      <c r="D13" t="s">
+        <v>1973</v>
+      </c>
+      <c r="E13" t="s">
+        <v>1974</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>91</v>
+      </c>
+      <c r="B14" t="s">
+        <v>1670</v>
+      </c>
+      <c r="C14" t="s">
+        <v>1878</v>
+      </c>
+      <c r="D14" t="s">
+        <v>1879</v>
+      </c>
+      <c r="E14" t="s">
+        <v>1880</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>95</v>
+      </c>
+      <c r="B15" t="s">
+        <v>429</v>
+      </c>
+      <c r="C15" t="s">
+        <v>1881</v>
+      </c>
+      <c r="D15" t="s">
+        <v>1882</v>
+      </c>
+      <c r="E15" t="s">
+        <v>1883</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>99</v>
+      </c>
+      <c r="B16" t="s">
+        <v>1884</v>
+      </c>
+      <c r="C16" t="s">
+        <v>1885</v>
+      </c>
+      <c r="D16" t="s">
+        <v>1977</v>
+      </c>
+      <c r="E16" t="s">
+        <v>1975</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>103</v>
+      </c>
+      <c r="B17" t="s">
+        <v>1876</v>
+      </c>
+      <c r="C17" t="s">
+        <v>1886</v>
+      </c>
+      <c r="D17" t="s">
+        <v>1978</v>
+      </c>
+      <c r="E17" t="s">
+        <v>1976</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>107</v>
+      </c>
+      <c r="B18" t="s">
+        <v>15</v>
+      </c>
+      <c r="C18" t="s">
+        <v>1887</v>
+      </c>
+      <c r="D18" t="s">
+        <v>1888</v>
+      </c>
+      <c r="E18" t="s">
+        <v>1889</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>111</v>
+      </c>
+      <c r="B19" t="s">
+        <v>1890</v>
+      </c>
+      <c r="C19" t="s">
+        <v>1891</v>
+      </c>
+      <c r="D19" t="s">
+        <v>1980</v>
+      </c>
+      <c r="E19" t="s">
+        <v>1979</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>115</v>
+      </c>
+      <c r="B20" t="s">
+        <v>1239</v>
+      </c>
+      <c r="C20" t="s">
+        <v>1892</v>
+      </c>
+      <c r="D20" t="s">
+        <v>1983</v>
+      </c>
+      <c r="E20" t="s">
+        <v>1981</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>119</v>
+      </c>
+      <c r="B21" t="s">
+        <v>1876</v>
+      </c>
+      <c r="C21" t="s">
+        <v>1893</v>
+      </c>
+      <c r="D21" t="s">
+        <v>1984</v>
+      </c>
+      <c r="E21" t="s">
+        <v>1982</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>123</v>
+      </c>
+      <c r="B22" t="s">
+        <v>681</v>
+      </c>
+      <c r="C22" t="s">
+        <v>1894</v>
+      </c>
+      <c r="D22" t="s">
+        <v>1895</v>
+      </c>
+      <c r="E22" t="s">
+        <v>1896</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>127</v>
+      </c>
+      <c r="B23" t="s">
+        <v>1807</v>
+      </c>
+      <c r="C23" t="s">
+        <v>1897</v>
+      </c>
+      <c r="D23" t="s">
+        <v>1898</v>
+      </c>
+      <c r="E23" t="s">
+        <v>1899</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>131</v>
+      </c>
+      <c r="B24" t="s">
+        <v>1844</v>
+      </c>
+      <c r="C24" t="s">
+        <v>1900</v>
+      </c>
+      <c r="D24" t="s">
+        <v>1901</v>
+      </c>
+      <c r="E24" t="s">
+        <v>1902</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>134</v>
+      </c>
+      <c r="B25" t="s">
+        <v>1752</v>
+      </c>
+      <c r="C25" t="s">
+        <v>1903</v>
+      </c>
+      <c r="D25" t="s">
+        <v>1904</v>
+      </c>
+      <c r="E25" t="s">
+        <v>1905</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>138</v>
+      </c>
+      <c r="B26" t="s">
+        <v>1701</v>
+      </c>
+      <c r="C26" t="s">
+        <v>1906</v>
+      </c>
+      <c r="D26" t="s">
+        <v>1907</v>
+      </c>
+      <c r="E26" t="s">
+        <v>1908</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>142</v>
+      </c>
+      <c r="B27" t="s">
+        <v>1769</v>
+      </c>
+      <c r="C27" t="s">
+        <v>1909</v>
+      </c>
+      <c r="D27" t="s">
+        <v>1910</v>
+      </c>
+      <c r="E27" t="s">
+        <v>1911</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>146</v>
+      </c>
+      <c r="B28" t="s">
+        <v>453</v>
+      </c>
+      <c r="C28" t="s">
+        <v>1912</v>
+      </c>
+      <c r="D28" t="s">
+        <v>1913</v>
+      </c>
+      <c r="E28" t="s">
+        <v>1914</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>150</v>
+      </c>
+      <c r="B29" t="s">
+        <v>1915</v>
+      </c>
+      <c r="C29" t="s">
+        <v>1916</v>
+      </c>
+      <c r="D29" t="s">
+        <v>1917</v>
+      </c>
+      <c r="E29" t="s">
+        <v>1918</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>154</v>
+      </c>
+      <c r="B30" t="s">
+        <v>1919</v>
+      </c>
+      <c r="C30" t="s">
+        <v>1920</v>
+      </c>
+      <c r="D30" t="s">
+        <v>1921</v>
+      </c>
+      <c r="E30" t="s">
+        <v>1922</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>158</v>
+      </c>
+      <c r="B31" t="s">
+        <v>1685</v>
+      </c>
+      <c r="C31" t="s">
+        <v>1923</v>
+      </c>
+      <c r="D31" t="s">
+        <v>1924</v>
+      </c>
+      <c r="E31" t="s">
+        <v>1925</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>162</v>
+      </c>
+      <c r="B32" t="s">
+        <v>1926</v>
+      </c>
+      <c r="C32" t="s">
+        <v>1927</v>
+      </c>
+      <c r="D32" t="s">
+        <v>1989</v>
+      </c>
+      <c r="E32" t="s">
+        <v>1990</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>166</v>
+      </c>
+      <c r="B33" t="s">
+        <v>1928</v>
+      </c>
+      <c r="C33" t="s">
+        <v>1929</v>
+      </c>
+      <c r="D33" t="s">
+        <v>1986</v>
+      </c>
+      <c r="E33" t="s">
+        <v>1985</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>171</v>
+      </c>
+      <c r="B34" t="s">
+        <v>1930</v>
+      </c>
+      <c r="C34" t="s">
+        <v>1931</v>
+      </c>
+      <c r="D34" t="s">
+        <v>1932</v>
+      </c>
+      <c r="E34" t="s">
+        <v>1933</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>175</v>
+      </c>
+      <c r="B35" t="s">
+        <v>504</v>
+      </c>
+      <c r="C35" t="s">
+        <v>1934</v>
+      </c>
+      <c r="D35" t="s">
+        <v>1935</v>
+      </c>
+      <c r="E35" t="s">
+        <v>1936</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>179</v>
+      </c>
+      <c r="B36" t="s">
+        <v>1701</v>
+      </c>
+      <c r="C36" t="s">
+        <v>1937</v>
+      </c>
+      <c r="D36" t="s">
+        <v>1938</v>
+      </c>
+      <c r="E36" t="s">
+        <v>1939</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>181</v>
+      </c>
+      <c r="B37" t="s">
+        <v>1876</v>
+      </c>
+      <c r="C37" t="s">
+        <v>1940</v>
+      </c>
+      <c r="D37" t="s">
+        <v>1941</v>
+      </c>
+      <c r="E37" t="s">
+        <v>1942</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>185</v>
+      </c>
+      <c r="B38" t="s">
+        <v>1943</v>
+      </c>
+      <c r="C38" t="s">
+        <v>1944</v>
+      </c>
+      <c r="D38" t="s">
+        <v>1945</v>
+      </c>
+      <c r="E38" t="s">
+        <v>1946</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>189</v>
+      </c>
+      <c r="B39" t="s">
+        <v>1947</v>
+      </c>
+      <c r="C39" t="s">
+        <v>1948</v>
+      </c>
+      <c r="D39" t="s">
+        <v>1949</v>
+      </c>
+      <c r="E39" t="s">
+        <v>1950</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>193</v>
+      </c>
+      <c r="B40" t="s">
+        <v>1951</v>
+      </c>
+      <c r="C40" t="s">
+        <v>1952</v>
+      </c>
+      <c r="D40" t="s">
+        <v>1953</v>
+      </c>
+      <c r="E40" t="s">
+        <v>1954</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>197</v>
+      </c>
+      <c r="B41" t="s">
+        <v>1876</v>
+      </c>
+      <c r="C41" t="s">
+        <v>1955</v>
+      </c>
+      <c r="D41" t="s">
+        <v>1956</v>
+      </c>
+      <c r="E41" t="s">
+        <v>1957</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>201</v>
+      </c>
+      <c r="B42" t="s">
+        <v>1712</v>
+      </c>
+      <c r="C42" t="s">
+        <v>1958</v>
+      </c>
+      <c r="D42" t="s">
+        <v>1959</v>
+      </c>
+      <c r="E42" t="s">
+        <v>1960</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>205</v>
+      </c>
+      <c r="B43" t="s">
+        <v>1740</v>
+      </c>
+      <c r="C43" t="s">
+        <v>1961</v>
+      </c>
+      <c r="D43" t="s">
+        <v>1962</v>
+      </c>
+      <c r="E43" t="s">
+        <v>1963</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>209</v>
+      </c>
+      <c r="B44" t="s">
+        <v>1964</v>
+      </c>
+      <c r="C44" t="s">
+        <v>1965</v>
+      </c>
+      <c r="D44" t="s">
+        <v>1988</v>
+      </c>
+      <c r="E44" t="s">
+        <v>1987</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>212</v>
+      </c>
+      <c r="B45" t="s">
+        <v>1681</v>
+      </c>
+      <c r="C45" t="s">
+        <v>1966</v>
+      </c>
+      <c r="D45" t="s">
+        <v>1967</v>
+      </c>
+      <c r="E45" t="s">
+        <v>1968</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:L44"/>
@@ -14829,12 +17878,6 @@
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="B29:B31"/>
-    <mergeCell ref="B14:B16"/>
-    <mergeCell ref="A8:A10"/>
-    <mergeCell ref="A26:A28"/>
-    <mergeCell ref="A17:A19"/>
-    <mergeCell ref="A20:A22"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A5:A7"/>
     <mergeCell ref="A23:A25"/>
@@ -14851,6 +17894,12 @@
     <mergeCell ref="B17:B19"/>
     <mergeCell ref="B23:B25"/>
     <mergeCell ref="A29:A31"/>
+    <mergeCell ref="B29:B31"/>
+    <mergeCell ref="B14:B16"/>
+    <mergeCell ref="A8:A10"/>
+    <mergeCell ref="A26:A28"/>
+    <mergeCell ref="A17:A19"/>
+    <mergeCell ref="A20:A22"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <ignoredErrors>

</xml_diff>

<commit_message>
Add GHOST secret monster system (25 forms): 5% evolve chance, 24 Evo2 branches, Overdrives, Echo Passives, new Blind status
</commit_message>
<xml_diff>
--- a/SYMBEAST_Evolve_Forms.xlsx
+++ b/SYMBEAST_Evolve_Forms.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\skyit\Desktop\Symbeast-main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B108191-F671-49A6-8113-83BAD93AB664}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34B510CA-2E55-47F7-A5AD-9F249BF4CEA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="11" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3608" uniqueCount="2127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3862" uniqueCount="2317">
   <si>
     <t>SYMBEAST — Evolved Forms (Stage 1, 10 forms)</t>
   </si>
@@ -6417,6 +6417,576 @@
   </si>
   <si>
     <t>Damage received -13%</t>
+  </si>
+  <si>
+    <t>GHOST</t>
+  </si>
+  <si>
+    <t>🌟</t>
+  </si>
+  <si>
+    <t>เมื่อเริ่มต่อสู้ สุ่มได้รับ 1 บัฟ: ATK+25%, โอกาสหลบ +25% หรือ DEF+25% (ตลอดการต่อสู้)</t>
+  </si>
+  <si>
+    <t>RAGEBEAR-GHOST</t>
+  </si>
+  <si>
+    <t>โจมตี x1.75 เมื่อศัตรูมี HP &gt; 70%</t>
+  </si>
+  <si>
+    <t>BEAR RAGE</t>
+  </si>
+  <si>
+    <t>โจมตี x4.0 + สตันเทิร์นนี้ จากนั้น ATK+30% และ Crit+25% นาน 3 เทิร์น</t>
+  </si>
+  <si>
+    <t>LION-GHOST</t>
+  </si>
+  <si>
+    <t>โจมตี 3 เทิร์นแรกใส่ศัตรูแต่ละตัวติดคริติคอลแน่นอน และลด ATK ศัตรู 10% ตลอดการต่อสู้</t>
+  </si>
+  <si>
+    <t>KING'S ROAR</t>
+  </si>
+  <si>
+    <t>โจมตี x3.5 จากนั้น ATK+40% และศัตรู DEF-20% นาน 3 เทิร์น</t>
+  </si>
+  <si>
+    <t>TIGER-GHOST</t>
+  </si>
+  <si>
+    <t>เมื่อ WIN ดาเมจ+50% เมื่อ LOSE SPD+100% ในรอบถัดไป</t>
+  </si>
+  <si>
+    <t>TIGER CLAW</t>
+  </si>
+  <si>
+    <t>โจมตี x4.0 ทะลุ DEF + คริติคอลแน่นอนเป็นเวลา 3 เทิร์น</t>
+  </si>
+  <si>
+    <t>WOLF-GHOST</t>
+  </si>
+  <si>
+    <t>โอกาสโจมตี 2 ครั้ง 25% เพิ่มเป็น 35% เมื่อ HP&lt;50%</t>
+  </si>
+  <si>
+    <t>WOLF FANG</t>
+  </si>
+  <si>
+    <t>โจมตี 2 ครั้ง x2.5 จากนั้นโอกาสโจมตี 2 ครั้ง +50% นาน 3 เทิร์น</t>
+  </si>
+  <si>
+    <t>SHARK-GHOST</t>
+  </si>
+  <si>
+    <t>ดาเมจ+30% ดูดเลือด 30% ใส่ศัตรูที่ HP&lt;50%</t>
+  </si>
+  <si>
+    <t>SHARK BITE</t>
+  </si>
+  <si>
+    <t>โจมตี x4.0 หากศัตรู HP&lt;50% หรือ x2.5 หาก HP&gt;50% จากนั้นดูดเลือด 25% นาน 3 เทิร์น</t>
+  </si>
+  <si>
+    <t>MANTIS-GHOST</t>
+  </si>
+  <si>
+    <t>ความแรงของดาเมจคริติคอล x2.0 แทน x1.6 และเมื่อ HP&lt;20% ดาเมจที่ทำได้ +50%</t>
+  </si>
+  <si>
+    <t>MANTIS SLASH</t>
+  </si>
+  <si>
+    <t>โจมตี x3.5 (คริบังคับ) + DEF ศัตรู -50% นาน 3 เทิร์น</t>
+  </si>
+  <si>
+    <t>BEE-GHOST</t>
+  </si>
+  <si>
+    <t>โอกาส 15% โจมตี 3 ครั้ง เมื่อสำเร็จมีโอกาสทำให้ศัตรูติดพิษ 50%</t>
+  </si>
+  <si>
+    <t>BEE SWARM</t>
+  </si>
+  <si>
+    <t>โจมตี 4 ครั้ง x1.5 จากนั้นหลบ+25% นาน 3 เทิร์น</t>
+  </si>
+  <si>
+    <t>BUNNY-GHOST</t>
+  </si>
+  <si>
+    <t>หลบ 20% เมื่อหลบสำเร็จ ATK+50% รอบถัดไป</t>
+  </si>
+  <si>
+    <t>BUNNY HOP</t>
+  </si>
+  <si>
+    <t>โจมตี x3.0 + หลบสมบูรณ์เทิร์นนี้ จากนั้นหลบ+35% และมีโอกาส 50% ทำให้ศัตรูติดสถานะตาบอด (โจมตีพลาด 50%) นาน 3 เทิร์น</t>
+  </si>
+  <si>
+    <t>TRICKFOX-GHOST</t>
+  </si>
+  <si>
+    <t>โอกาส 50% ทำให้ศัตรูติดสถานะเผาไหม้ เป็นเวลา 3 เทิร์น</t>
+  </si>
+  <si>
+    <t>FOX TRICK</t>
+  </si>
+  <si>
+    <t>โจมตี x3.0 + ทำให้ศัตรูติดสถานะฟื้นฟู HP ไม่ได้ 3 เทิร์น จากนั้นหลบ+25% นาน 3 เทิร์น</t>
+  </si>
+  <si>
+    <t>OWL-GHOST</t>
+  </si>
+  <si>
+    <t>โจมตีไม่พลาดเป้า และมีโอกาส 15% ทำให้ศัตรูติดสถานะตาบอด (โจมตีพลาด 50% เป็นเวลา 3 เทิร์น)</t>
+  </si>
+  <si>
+    <t>OWL SIGHT</t>
+  </si>
+  <si>
+    <t>โจมตี x3.0 (ติดคริติคอล) + จากนั้น ATK/SPD+25% นาน 3 เทิร์น</t>
+  </si>
+  <si>
+    <t>VOLTMOUSE-GHOST</t>
+  </si>
+  <si>
+    <t>ทุกเทิร์นมีโอกาสสุ่ม ทำให้ศัตรูสตัน, ลด ATK 50%, ลด DEF 50%, เพิ่ม ATK 25%(ให้ศัตรู)</t>
+  </si>
+  <si>
+    <t>THUNDER SHOCK</t>
+  </si>
+  <si>
+    <t>โจมตี x3.0 + สตันเทิร์นนี้ จากนั้น SPDx2.0 และโอกาสสตัน+30% นาน 3 เทิร์น</t>
+  </si>
+  <si>
+    <t>PENGUIN-GHOST</t>
+  </si>
+  <si>
+    <t>ลดดาเมจ 15% เมื่อ HP&lt;50% หลบ+25% ATK+25%</t>
+  </si>
+  <si>
+    <t>ICE SLIDE</t>
+  </si>
+  <si>
+    <t>โจมตี x3.5 + หลบสมบูรณ์เทิร์นนี้ + DEF+50% นาน 3 เทิร์น</t>
+  </si>
+  <si>
+    <t>COCKROACH-GHOST</t>
+  </si>
+  <si>
+    <t>เมื่อถูกโจมตีถึงตายจะเหลือ HP 1 (1 ครั้ง/การต่อสู้) และ DEF/SPD+100% ตลอดการต่อสู้นั้น</t>
+  </si>
+  <si>
+    <t>ROACH SURVIVAL</t>
+  </si>
+  <si>
+    <t>รับดาเมจ 1 เทิร์นนี้ + ฟื้น HP 30% จากนั้นลดดาเมจ 25% และมีโอกาส 50% ทำให้ศัตรูติดสถานะตาบอด (โจมตีพลาด 50%) นาน 3 เทิร์น</t>
+  </si>
+  <si>
+    <t>SLIME-GHOST</t>
+  </si>
+  <si>
+    <t>ฟื้น HP 5% ทุกรอบ และเมื่อถูกโจมตีหรือโจมตีศัตรูมีโอกาส 25% ทำให้ศัตรูติดพิษ</t>
+  </si>
+  <si>
+    <t>SLIME ABSORB</t>
+  </si>
+  <si>
+    <t>ดูด HP ศัตรู 25% + ฟื้น HP 30% จากนั้นฟื้น 10% ต่อเทิร์น นาน 3 เทิร์น</t>
+  </si>
+  <si>
+    <t>LEAPFROG-GHOST</t>
+  </si>
+  <si>
+    <t>โอกาส 25% สะท้อนดาเมจ 50% และทำให้ศัตรูติดพิษ</t>
+  </si>
+  <si>
+    <t>FROG LEAP</t>
+  </si>
+  <si>
+    <t>โจมตี x2.5 + สะท้อนดาเมจ 100% เทิร์นนี้ จากนั้นสะท้อน 50% + ATK+25% นาน 3 เทิร์น</t>
+  </si>
+  <si>
+    <t>HAMSTER-GHOST</t>
+  </si>
+  <si>
+    <t>ทุก 3 เทิร์นฟื้น HP 20% และ DEF+50% ในรอบนั้น</t>
+  </si>
+  <si>
+    <t>HAMSTER STASH</t>
+  </si>
+  <si>
+    <t>รับดาเมจ 1 เทิร์นนี้ + ฟื้น HP 40% จากนั้น DEF+30% + ฟื้น 8% ต่อเทิร์น 3 เทิร์น</t>
+  </si>
+  <si>
+    <t>AXOLOTL-GHOST</t>
+  </si>
+  <si>
+    <t>เมื่อถูกโจมตีโอกาส 30% ฟื้น HP 15%</t>
+  </si>
+  <si>
+    <t>AXOLOTL REGEN</t>
+  </si>
+  <si>
+    <t>โจมตี x2.0 + ฟื้น HP 50% และล้างสถานะผิดปกติทั้งหมด จากนั้นฟื้น 12% ต่อเทิร์น นาน 3 เทิร์น</t>
+  </si>
+  <si>
+    <t>CAT-GHOST</t>
+  </si>
+  <si>
+    <t>หลบ 25% ถ้าโดนโจมตี รอบถัดไปจะ ATK+50%</t>
+  </si>
+  <si>
+    <t>CAT NINE LIVES</t>
+  </si>
+  <si>
+    <t>โจมตี x3.0 + หลบสมบูรณ์เทิร์นนี้ จากนั้นหลบ+30% + ATK+50% นาน 3 เทิร์น</t>
+  </si>
+  <si>
+    <t>DRAGON-GHOST</t>
+  </si>
+  <si>
+    <t>ATK/DEF/SPD +3% ทุกรอบ (สูงสุด 10 ครั้ง) และมีโอกาส 15% ทำให้ศัตรูติดสถานะเผาไหม้ เป็นเวลา 3 เทิร์น</t>
+  </si>
+  <si>
+    <t>DRAGON BREATH</t>
+  </si>
+  <si>
+    <t>โจมตี x3.5 + ทำให้ศัตรูติดสถานะเผาไหม้ จากนั้น ATK/DEF/SPD+20% นาน 3 เทิร์น</t>
+  </si>
+  <si>
+    <t>GRIFFON-GHOST</t>
+  </si>
+  <si>
+    <t>หลบ 15%, Crit Rate+15% เมื่อโจมตีติดคริติคอล จะทำให้ศัตรูติดสถานะฟื้นฟู HP ไม่ได้ 3 เทิร์น</t>
+  </si>
+  <si>
+    <t>GRIFFON DIVE</t>
+  </si>
+  <si>
+    <t>โจมตี x3.5 ทะลุ DEF + หลบเทิร์นนี้ จากนั้น ATK/SPD+30% นาน 3 เทิร์น</t>
+  </si>
+  <si>
+    <t>OCTOPUS-GHOST</t>
+  </si>
+  <si>
+    <t>โอกาส 30% ทำให้ศัตรูติดสถานะตาบอด (โจมตีพลาด 50% เป็นเวลา 3 เทิร์น)</t>
+  </si>
+  <si>
+    <t>OCTOPUS INK</t>
+  </si>
+  <si>
+    <t>โจมตี x2.5 + ศัตรูตาบอด (โจมตีพลาด 50%) 3 เทิร์น จากนั้น ATK+25% นาน 3 เทิร์น</t>
+  </si>
+  <si>
+    <t>PHOENIX-GHOST</t>
+  </si>
+  <si>
+    <t>เมื่อตายจะฟื้นคืนชีพด้วย HP 50% และทำให้ศัตรูติดสถานะเผาไหม้ 10 เทิร์น (1 ครั้ง/การต่อสู้)</t>
+  </si>
+  <si>
+    <t>PHOENIX REBIRTH</t>
+  </si>
+  <si>
+    <t>โจมตี x3.5 + ฟื้น HP 25% จากนั้น ATK/SPD+30% นาน 3 เทิร์น</t>
+  </si>
+  <si>
+    <t>UNICORN-GHOST</t>
+  </si>
+  <si>
+    <t>ฟื้น HP 8% ต่อเทิร์น ล้างดีบัฟ 1 อย่างต่อเทิร์น (Curse/No-Heal/Burn/Poison/Stun/Blind/Heal-Block — ครอบคลุมทุกประเภท)</t>
+  </si>
+  <si>
+    <t>UNICORN BLESS</t>
+  </si>
+  <si>
+    <t>โจมตี x3.0 + ฟื้น 40% + ล้างสถานะทั้งหมด จากนั้น ATK/SPD/DEF+20% + ฟื้น 10% ต่อเทิร์น 3 เทิร์น</t>
+  </si>
+  <si>
+    <t>PANDA-GHOST</t>
+  </si>
+  <si>
+    <t>Crit Rate+25% โอกาสสตัน 15% เมื่อโจมตี</t>
+  </si>
+  <si>
+    <t>PANDA STRIKE</t>
+  </si>
+  <si>
+    <t>โจมตี x4 (คริบังคับ) + สตัน จากนั้น Crit+30% + โอกาสสตัน+20% นาน 3 เทิร์น</t>
+  </si>
+  <si>
+    <t>RAGE ECHO</t>
+  </si>
+  <si>
+    <t>Damage +35% when enemy HP &gt; 70%</t>
+  </si>
+  <si>
+    <t>ดาเมจ +35% เมื่อศัตรูมี HP &gt; 70%</t>
+  </si>
+  <si>
+    <t>ROAR ECHO</t>
+  </si>
+  <si>
+    <t>First 3 turns: crit chance +50% and permanently reduce enemy ATK by 5%</t>
+  </si>
+  <si>
+    <t>3 เทิร์นแรก: โอกาสคริ +50% และลด ATK ศัตรู 5% ตลอดการต่อสู้</t>
+  </si>
+  <si>
+    <t>🐯</t>
+  </si>
+  <si>
+    <t>TIGER ECHO</t>
+  </si>
+  <si>
+    <t>On WIN: damage +25%; on LOSE: SPD+50% next round</t>
+  </si>
+  <si>
+    <t>เมื่อ WIN: ดาเมจ+25% เมื่อ LOSE: SPD+50% รอบถัดไป</t>
+  </si>
+  <si>
+    <t>WOLF ECHO</t>
+  </si>
+  <si>
+    <t>12% chance to attack twice (20% when HP&lt;50%)</t>
+  </si>
+  <si>
+    <t>โอกาส 12% โจมตี 2 ครั้ง (20% เมื่อ HP&lt;50%)</t>
+  </si>
+  <si>
+    <t>🦈</t>
+  </si>
+  <si>
+    <t>SHARK ECHO</t>
+  </si>
+  <si>
+    <t>+15% damage and 15% lifesteal vs enemies with HP&lt;50%</t>
+  </si>
+  <si>
+    <t>ดาเมจ+15% และดูดเลือด 15% ใส่ศัตรู HP&lt;50%</t>
+  </si>
+  <si>
+    <t>MANTIS ECHO</t>
+  </si>
+  <si>
+    <t>Crit damage x2. When HP&lt;20%: damage +25%</t>
+  </si>
+  <si>
+    <t>คริติคอลดาเมจ x2 เมื่อ HP&lt;20%: ดาเมจ+25%</t>
+  </si>
+  <si>
+    <t>🐝</t>
+  </si>
+  <si>
+    <t>SWARM ECHO</t>
+  </si>
+  <si>
+    <t>10% chance to attack 3 times; on success, 25% chance to poison enemy</t>
+  </si>
+  <si>
+    <t>โอกาส 10% โจมตี 3 ครั้ง เมื่อสำเร็จ โอกาส 25% ทำให้ศัตรูติดพิษ</t>
+  </si>
+  <si>
+    <t>🐰</t>
+  </si>
+  <si>
+    <t>BUNNY ECHO</t>
+  </si>
+  <si>
+    <t>10% dodge; on dodge: ATK+25% next round</t>
+  </si>
+  <si>
+    <t>หลบ 10% เมื่อหลบสำเร็จ ATK+25% รอบถัดไป</t>
+  </si>
+  <si>
+    <t>🎭</t>
+  </si>
+  <si>
+    <t>TRICK ECHO</t>
+  </si>
+  <si>
+    <t>25% chance to Burn the enemy for 3 turns</t>
+  </si>
+  <si>
+    <t>โอกาส 25% ทำให้ศัตรูติดสถานะเผาไหม้ 3 เทิร์น</t>
+  </si>
+  <si>
+    <t>👁️</t>
+  </si>
+  <si>
+    <t>OWL ECHO</t>
+  </si>
+  <si>
+    <t>Attacks never miss; 10% chance to Blind enemy on hit</t>
+  </si>
+  <si>
+    <t>โจมตีไม่พลาดเป้า โอกาส 10% ทำให้ศัตรูตาบอดเมื่อโจมตี</t>
+  </si>
+  <si>
+    <t>VOLT ECHO</t>
+  </si>
+  <si>
+    <t>Every turn: random effect — stun enemy, ATK-50%, DEF-50%, or give enemy ATK+25%</t>
+  </si>
+  <si>
+    <t>ทุกเทิร์นมีโอกาสสุ่ม ทำให้ศัตรูสตัน,ลด ATK 50%,ลด DEF 50%, เพิ่ม ATK 25%(ให้ศัตรู)</t>
+  </si>
+  <si>
+    <t>🐧</t>
+  </si>
+  <si>
+    <t>PENGUIN ECHO</t>
+  </si>
+  <si>
+    <t>Damage taken -10%; when HP&lt;50%: dodge+10% and ATK+15%</t>
+  </si>
+  <si>
+    <t>ลดดาเมจ 10% เมื่อ HP&lt;50%: หลบ+10% และ ATK+15%</t>
+  </si>
+  <si>
+    <t>🪳</t>
+  </si>
+  <si>
+    <t>ROACH ECHO</t>
+  </si>
+  <si>
+    <t>Survive a fatal blow with 1 HP (once), then DEF/SPD+50% for rest of battle</t>
+  </si>
+  <si>
+    <t>เหลือ HP 1 เมื่อถูกโจมตีถึงตาย (1 ครั้ง) จากนั้น DEF/SPD+50% ตลอดการต่อสู้</t>
+  </si>
+  <si>
+    <t>🟢</t>
+  </si>
+  <si>
+    <t>OOZE ECHO</t>
+  </si>
+  <si>
+    <t>Recover 3% HP/round; 15% chance to poison on attack or when hit</t>
+  </si>
+  <si>
+    <t>ฟื้น HP 3% ทุกรอบ โอกาส 15% ทำให้ศัตรูติดพิษเมื่อโจมตีหรือถูกโจมตี</t>
+  </si>
+  <si>
+    <t>💦</t>
+  </si>
+  <si>
+    <t>FROG ECHO</t>
+  </si>
+  <si>
+    <t>15% chance to reflect 25% damage and poison the enemy</t>
+  </si>
+  <si>
+    <t>โอกาส 15% สะท้อนดาเมจ 25% และทำให้ศัตรูติดพิษ</t>
+  </si>
+  <si>
+    <t>🐹</t>
+  </si>
+  <si>
+    <t>HAMSTER ECHO</t>
+  </si>
+  <si>
+    <t>Every 3 turns: recover 10% HP and DEF+25% that round</t>
+  </si>
+  <si>
+    <t>ทุก 3 เทิร์น: ฟื้น HP 10% และ DEF+25% ในรอบนั้น</t>
+  </si>
+  <si>
+    <t>🦎</t>
+  </si>
+  <si>
+    <t>AXOLOTL ECHO</t>
+  </si>
+  <si>
+    <t>15% chance to recover 8% HP when hit</t>
+  </si>
+  <si>
+    <t>โอกาส 15% ฟื้น HP 8% เมื่อถูกโจมตี</t>
+  </si>
+  <si>
+    <t>😼</t>
+  </si>
+  <si>
+    <t>CAT ECHO</t>
+  </si>
+  <si>
+    <t>15% dodge; if hit: ATK+25% next round</t>
+  </si>
+  <si>
+    <t>หลบ 15% ถ้าโดนโจมตี: ATK+25% รอบถัดไป</t>
+  </si>
+  <si>
+    <t>DRAGON ECHO</t>
+  </si>
+  <si>
+    <t>ATK/DEF/SPD +1.5%/round (max 10 stacks); 8% chance to Burn enemy</t>
+  </si>
+  <si>
+    <t>ATK/DEF/SPD +1.5% ต่อรอบ (สูงสุด 10 ครั้ง) โอกาส 8% เผาศัตรู</t>
+  </si>
+  <si>
+    <t>GRIFFON ECHO</t>
+  </si>
+  <si>
+    <t>10% dodge, 10% crit; on crit: enemy cannot heal for 3 turns</t>
+  </si>
+  <si>
+    <t>หลบ 10%, Crit+10% เมื่อคริ: ศัตรูฟื้นฟู HP ไม่ได้ 3 เทิร์น</t>
+  </si>
+  <si>
+    <t>🐙</t>
+  </si>
+  <si>
+    <t>OCTOPUS ECHO</t>
+  </si>
+  <si>
+    <t>15% chance to Blind enemy on hit (50% miss for 3 turns)</t>
+  </si>
+  <si>
+    <t>โอกาส 15% ทำให้ศัตรูตาบอด (โจมตีพลาด 50% 3 เทิร์น)</t>
+  </si>
+  <si>
+    <t>🔱</t>
+  </si>
+  <si>
+    <t>Once: revive with 25% HP, Burn enemy for 5 turns</t>
+  </si>
+  <si>
+    <t>ครั้งเดียว: ฟื้นคืนชีพด้วย HP 25% เผาศัตรู 5 เทิร์น</t>
+  </si>
+  <si>
+    <t>UNICORN ECHO</t>
+  </si>
+  <si>
+    <t>Recover 4% HP/turn; cleanse 1 debuff every turn (covers all debuff types)</t>
+  </si>
+  <si>
+    <t>ฟื้น HP 4% ต่อเทิร์น ล้างดีบัฟ 1 อย่างต่อเทิร์น (ครอบคลุมทุกประเภท)</t>
+  </si>
+  <si>
+    <t>PANDA ECHO</t>
+  </si>
+  <si>
+    <t>Crit+15%; 10% chance to stun on hit</t>
+  </si>
+  <si>
+    <t>Crit+15% โอกาสสตัน 10% เมื่อโจมตี</t>
+  </si>
+  <si>
+    <t>blind_gaze</t>
+  </si>
+  <si>
+    <t>BLIND GAZE</t>
+  </si>
+  <si>
+    <t>จ้องตาบอด</t>
+  </si>
+  <si>
+    <t>20% chance to blind you on a landed hit (50% miss chance for 3 turns)</t>
+  </si>
+  <si>
+    <t>20% โอกาสทำให้ผู้เล่นตาบอดเมื่อโจมตีโดน (โจมตีพลาด 50% นาน 3 เทิร์น)</t>
   </si>
 </sst>
 </file>
@@ -6795,7 +7365,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
@@ -7106,6 +7676,32 @@
       </c>
       <c r="H14" t="s">
         <v>48</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>2127</v>
+      </c>
+      <c r="B15" t="s">
+        <v>2128</v>
+      </c>
+      <c r="C15" t="s">
+        <v>2127</v>
+      </c>
+      <c r="D15">
+        <v>75</v>
+      </c>
+      <c r="E15">
+        <v>20</v>
+      </c>
+      <c r="F15">
+        <v>16</v>
+      </c>
+      <c r="G15">
+        <v>10</v>
+      </c>
+      <c r="H15" t="s">
+        <v>2129</v>
       </c>
     </row>
   </sheetData>
@@ -15774,7 +16370,7 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F00FD1CF-924F-4FD0-B28B-32154B63F96A}">
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E69"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.69921875" customWidth="1"/>
@@ -16493,6 +17089,414 @@
       </c>
       <c r="E45" t="s">
         <v>1968</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>2130</v>
+      </c>
+      <c r="B46" t="s">
+        <v>1662</v>
+      </c>
+      <c r="C46" t="s">
+        <v>2226</v>
+      </c>
+      <c r="D46" t="s">
+        <v>2227</v>
+      </c>
+      <c r="E46" t="s">
+        <v>2228</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>2134</v>
+      </c>
+      <c r="B47" t="s">
+        <v>1807</v>
+      </c>
+      <c r="C47" t="s">
+        <v>2229</v>
+      </c>
+      <c r="D47" t="s">
+        <v>2230</v>
+      </c>
+      <c r="E47" t="s">
+        <v>2231</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>2138</v>
+      </c>
+      <c r="B48" t="s">
+        <v>2232</v>
+      </c>
+      <c r="C48" t="s">
+        <v>2233</v>
+      </c>
+      <c r="D48" t="s">
+        <v>2234</v>
+      </c>
+      <c r="E48" t="s">
+        <v>2235</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>2142</v>
+      </c>
+      <c r="B49" t="s">
+        <v>1773</v>
+      </c>
+      <c r="C49" t="s">
+        <v>2236</v>
+      </c>
+      <c r="D49" t="s">
+        <v>2237</v>
+      </c>
+      <c r="E49" t="s">
+        <v>2238</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>2146</v>
+      </c>
+      <c r="B50" t="s">
+        <v>2239</v>
+      </c>
+      <c r="C50" t="s">
+        <v>2240</v>
+      </c>
+      <c r="D50" t="s">
+        <v>2241</v>
+      </c>
+      <c r="E50" t="s">
+        <v>2242</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>2150</v>
+      </c>
+      <c r="B51" t="s">
+        <v>681</v>
+      </c>
+      <c r="C51" t="s">
+        <v>2243</v>
+      </c>
+      <c r="D51" t="s">
+        <v>2244</v>
+      </c>
+      <c r="E51" t="s">
+        <v>2245</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>2154</v>
+      </c>
+      <c r="B52" t="s">
+        <v>2246</v>
+      </c>
+      <c r="C52" t="s">
+        <v>2247</v>
+      </c>
+      <c r="D52" t="s">
+        <v>2248</v>
+      </c>
+      <c r="E52" t="s">
+        <v>2249</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>2158</v>
+      </c>
+      <c r="B53" t="s">
+        <v>2250</v>
+      </c>
+      <c r="C53" t="s">
+        <v>2251</v>
+      </c>
+      <c r="D53" t="s">
+        <v>2252</v>
+      </c>
+      <c r="E53" t="s">
+        <v>2253</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>2162</v>
+      </c>
+      <c r="B54" t="s">
+        <v>2254</v>
+      </c>
+      <c r="C54" t="s">
+        <v>2255</v>
+      </c>
+      <c r="D54" t="s">
+        <v>2256</v>
+      </c>
+      <c r="E54" t="s">
+        <v>2257</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>2166</v>
+      </c>
+      <c r="B55" t="s">
+        <v>2258</v>
+      </c>
+      <c r="C55" t="s">
+        <v>2259</v>
+      </c>
+      <c r="D55" t="s">
+        <v>2260</v>
+      </c>
+      <c r="E55" t="s">
+        <v>2261</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>2170</v>
+      </c>
+      <c r="B56" t="s">
+        <v>15</v>
+      </c>
+      <c r="C56" t="s">
+        <v>2262</v>
+      </c>
+      <c r="D56" t="s">
+        <v>2263</v>
+      </c>
+      <c r="E56" t="s">
+        <v>2264</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
+        <v>2174</v>
+      </c>
+      <c r="B57" t="s">
+        <v>2265</v>
+      </c>
+      <c r="C57" t="s">
+        <v>2266</v>
+      </c>
+      <c r="D57" t="s">
+        <v>2267</v>
+      </c>
+      <c r="E57" t="s">
+        <v>2268</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>2178</v>
+      </c>
+      <c r="B58" t="s">
+        <v>2269</v>
+      </c>
+      <c r="C58" t="s">
+        <v>2270</v>
+      </c>
+      <c r="D58" t="s">
+        <v>2271</v>
+      </c>
+      <c r="E58" t="s">
+        <v>2272</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>2182</v>
+      </c>
+      <c r="B59" t="s">
+        <v>2273</v>
+      </c>
+      <c r="C59" t="s">
+        <v>2274</v>
+      </c>
+      <c r="D59" t="s">
+        <v>2275</v>
+      </c>
+      <c r="E59" t="s">
+        <v>2276</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
+        <v>2186</v>
+      </c>
+      <c r="B60" t="s">
+        <v>2277</v>
+      </c>
+      <c r="C60" t="s">
+        <v>2278</v>
+      </c>
+      <c r="D60" t="s">
+        <v>2279</v>
+      </c>
+      <c r="E60" t="s">
+        <v>2280</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
+        <v>2190</v>
+      </c>
+      <c r="B61" t="s">
+        <v>2281</v>
+      </c>
+      <c r="C61" t="s">
+        <v>2282</v>
+      </c>
+      <c r="D61" t="s">
+        <v>2283</v>
+      </c>
+      <c r="E61" t="s">
+        <v>2284</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A62" t="s">
+        <v>2194</v>
+      </c>
+      <c r="B62" t="s">
+        <v>2285</v>
+      </c>
+      <c r="C62" t="s">
+        <v>2286</v>
+      </c>
+      <c r="D62" t="s">
+        <v>2287</v>
+      </c>
+      <c r="E62" t="s">
+        <v>2288</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A63" t="s">
+        <v>2198</v>
+      </c>
+      <c r="B63" t="s">
+        <v>2289</v>
+      </c>
+      <c r="C63" t="s">
+        <v>2290</v>
+      </c>
+      <c r="D63" t="s">
+        <v>2291</v>
+      </c>
+      <c r="E63" t="s">
+        <v>2292</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A64" t="s">
+        <v>2202</v>
+      </c>
+      <c r="B64" t="s">
+        <v>1701</v>
+      </c>
+      <c r="C64" t="s">
+        <v>2293</v>
+      </c>
+      <c r="D64" t="s">
+        <v>2294</v>
+      </c>
+      <c r="E64" t="s">
+        <v>2295</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A65" t="s">
+        <v>2206</v>
+      </c>
+      <c r="B65" t="s">
+        <v>1693</v>
+      </c>
+      <c r="C65" t="s">
+        <v>2296</v>
+      </c>
+      <c r="D65" t="s">
+        <v>2297</v>
+      </c>
+      <c r="E65" t="s">
+        <v>2298</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A66" t="s">
+        <v>2210</v>
+      </c>
+      <c r="B66" t="s">
+        <v>2299</v>
+      </c>
+      <c r="C66" t="s">
+        <v>2300</v>
+      </c>
+      <c r="D66" t="s">
+        <v>2301</v>
+      </c>
+      <c r="E66" t="s">
+        <v>2302</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A67" t="s">
+        <v>2214</v>
+      </c>
+      <c r="B67" t="s">
+        <v>2303</v>
+      </c>
+      <c r="C67" t="s">
+        <v>1937</v>
+      </c>
+      <c r="D67" t="s">
+        <v>2304</v>
+      </c>
+      <c r="E67" t="s">
+        <v>2305</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A68" t="s">
+        <v>2218</v>
+      </c>
+      <c r="B68" t="s">
+        <v>589</v>
+      </c>
+      <c r="C68" t="s">
+        <v>2306</v>
+      </c>
+      <c r="D68" t="s">
+        <v>2307</v>
+      </c>
+      <c r="E68" t="s">
+        <v>2308</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A69" t="s">
+        <v>2222</v>
+      </c>
+      <c r="B69" t="s">
+        <v>1861</v>
+      </c>
+      <c r="C69" t="s">
+        <v>2309</v>
+      </c>
+      <c r="D69" t="s">
+        <v>2310</v>
+      </c>
+      <c r="E69" t="s">
+        <v>2311</v>
       </c>
     </row>
   </sheetData>
@@ -17875,7 +18879,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:L44"/>
+  <dimension ref="A1:L68"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="46.69921875" bestFit="1" customWidth="1"/>
@@ -19178,6 +20182,711 @@
       </c>
       <c r="L44" t="s">
         <v>215</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>2127</v>
+      </c>
+      <c r="B45" t="s">
+        <v>2127</v>
+      </c>
+      <c r="C45" t="s">
+        <v>2129</v>
+      </c>
+      <c r="D45" t="s">
+        <v>58</v>
+      </c>
+      <c r="E45" t="s">
+        <v>2130</v>
+      </c>
+      <c r="F45">
+        <v>112</v>
+      </c>
+      <c r="G45">
+        <v>48</v>
+      </c>
+      <c r="H45">
+        <v>15</v>
+      </c>
+      <c r="I45">
+        <v>6</v>
+      </c>
+      <c r="J45" t="s">
+        <v>2131</v>
+      </c>
+      <c r="K45" t="s">
+        <v>2132</v>
+      </c>
+      <c r="L45" t="s">
+        <v>2133</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="D46" t="s">
+        <v>58</v>
+      </c>
+      <c r="E46" t="s">
+        <v>2134</v>
+      </c>
+      <c r="F46">
+        <v>108</v>
+      </c>
+      <c r="G46">
+        <v>52</v>
+      </c>
+      <c r="H46">
+        <v>16</v>
+      </c>
+      <c r="I46">
+        <v>5</v>
+      </c>
+      <c r="J46" t="s">
+        <v>2135</v>
+      </c>
+      <c r="K46" t="s">
+        <v>2136</v>
+      </c>
+      <c r="L46" t="s">
+        <v>2137</v>
+      </c>
+    </row>
+    <row r="47" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="D47" t="s">
+        <v>58</v>
+      </c>
+      <c r="E47" t="s">
+        <v>2138</v>
+      </c>
+      <c r="F47">
+        <v>114</v>
+      </c>
+      <c r="G47">
+        <v>50</v>
+      </c>
+      <c r="H47">
+        <v>18</v>
+      </c>
+      <c r="I47">
+        <v>5</v>
+      </c>
+      <c r="J47" t="s">
+        <v>2139</v>
+      </c>
+      <c r="K47" t="s">
+        <v>2140</v>
+      </c>
+      <c r="L47" t="s">
+        <v>2141</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="D48" t="s">
+        <v>58</v>
+      </c>
+      <c r="E48" t="s">
+        <v>2142</v>
+      </c>
+      <c r="F48">
+        <v>106</v>
+      </c>
+      <c r="G48">
+        <v>46</v>
+      </c>
+      <c r="H48">
+        <v>20</v>
+      </c>
+      <c r="I48">
+        <v>6</v>
+      </c>
+      <c r="J48" t="s">
+        <v>2143</v>
+      </c>
+      <c r="K48" t="s">
+        <v>2144</v>
+      </c>
+      <c r="L48" t="s">
+        <v>2145</v>
+      </c>
+    </row>
+    <row r="49" spans="4:12" x14ac:dyDescent="0.3">
+      <c r="D49" t="s">
+        <v>58</v>
+      </c>
+      <c r="E49" t="s">
+        <v>2146</v>
+      </c>
+      <c r="F49">
+        <v>118</v>
+      </c>
+      <c r="G49">
+        <v>49</v>
+      </c>
+      <c r="H49">
+        <v>14</v>
+      </c>
+      <c r="I49">
+        <v>7</v>
+      </c>
+      <c r="J49" t="s">
+        <v>2147</v>
+      </c>
+      <c r="K49" t="s">
+        <v>2148</v>
+      </c>
+      <c r="L49" t="s">
+        <v>2149</v>
+      </c>
+    </row>
+    <row r="50" spans="4:12" x14ac:dyDescent="0.3">
+      <c r="D50" t="s">
+        <v>58</v>
+      </c>
+      <c r="E50" t="s">
+        <v>2150</v>
+      </c>
+      <c r="F50">
+        <v>102</v>
+      </c>
+      <c r="G50">
+        <v>54</v>
+      </c>
+      <c r="H50">
+        <v>17</v>
+      </c>
+      <c r="I50">
+        <v>4</v>
+      </c>
+      <c r="J50" t="s">
+        <v>2151</v>
+      </c>
+      <c r="K50" t="s">
+        <v>2152</v>
+      </c>
+      <c r="L50" t="s">
+        <v>2153</v>
+      </c>
+    </row>
+    <row r="51" spans="4:12" x14ac:dyDescent="0.3">
+      <c r="D51" t="s">
+        <v>63</v>
+      </c>
+      <c r="E51" t="s">
+        <v>2154</v>
+      </c>
+      <c r="F51">
+        <v>100</v>
+      </c>
+      <c r="G51">
+        <v>28</v>
+      </c>
+      <c r="H51">
+        <v>44</v>
+      </c>
+      <c r="I51">
+        <v>5</v>
+      </c>
+      <c r="J51" t="s">
+        <v>2155</v>
+      </c>
+      <c r="K51" t="s">
+        <v>2156</v>
+      </c>
+      <c r="L51" t="s">
+        <v>2157</v>
+      </c>
+    </row>
+    <row r="52" spans="4:12" x14ac:dyDescent="0.3">
+      <c r="D52" t="s">
+        <v>63</v>
+      </c>
+      <c r="E52" t="s">
+        <v>2158</v>
+      </c>
+      <c r="F52">
+        <v>96</v>
+      </c>
+      <c r="G52">
+        <v>24</v>
+      </c>
+      <c r="H52">
+        <v>48</v>
+      </c>
+      <c r="I52">
+        <v>4</v>
+      </c>
+      <c r="J52" t="s">
+        <v>2159</v>
+      </c>
+      <c r="K52" t="s">
+        <v>2160</v>
+      </c>
+      <c r="L52" t="s">
+        <v>2161</v>
+      </c>
+    </row>
+    <row r="53" spans="4:12" x14ac:dyDescent="0.3">
+      <c r="D53" t="s">
+        <v>63</v>
+      </c>
+      <c r="E53" t="s">
+        <v>2162</v>
+      </c>
+      <c r="F53">
+        <v>104</v>
+      </c>
+      <c r="G53">
+        <v>30</v>
+      </c>
+      <c r="H53">
+        <v>42</v>
+      </c>
+      <c r="I53">
+        <v>5</v>
+      </c>
+      <c r="J53" t="s">
+        <v>2163</v>
+      </c>
+      <c r="K53" t="s">
+        <v>2164</v>
+      </c>
+      <c r="L53" t="s">
+        <v>2165</v>
+      </c>
+    </row>
+    <row r="54" spans="4:12" x14ac:dyDescent="0.3">
+      <c r="D54" t="s">
+        <v>63</v>
+      </c>
+      <c r="E54" t="s">
+        <v>2166</v>
+      </c>
+      <c r="F54">
+        <v>108</v>
+      </c>
+      <c r="G54">
+        <v>26</v>
+      </c>
+      <c r="H54">
+        <v>40</v>
+      </c>
+      <c r="I54">
+        <v>6</v>
+      </c>
+      <c r="J54" t="s">
+        <v>2167</v>
+      </c>
+      <c r="K54" t="s">
+        <v>2168</v>
+      </c>
+      <c r="L54" t="s">
+        <v>2169</v>
+      </c>
+    </row>
+    <row r="55" spans="4:12" x14ac:dyDescent="0.3">
+      <c r="D55" t="s">
+        <v>63</v>
+      </c>
+      <c r="E55" t="s">
+        <v>2170</v>
+      </c>
+      <c r="F55">
+        <v>98</v>
+      </c>
+      <c r="G55">
+        <v>32</v>
+      </c>
+      <c r="H55">
+        <v>46</v>
+      </c>
+      <c r="I55">
+        <v>4</v>
+      </c>
+      <c r="J55" t="s">
+        <v>2171</v>
+      </c>
+      <c r="K55" t="s">
+        <v>2172</v>
+      </c>
+      <c r="L55" t="s">
+        <v>2173</v>
+      </c>
+    </row>
+    <row r="56" spans="4:12" x14ac:dyDescent="0.3">
+      <c r="D56" t="s">
+        <v>63</v>
+      </c>
+      <c r="E56" t="s">
+        <v>2174</v>
+      </c>
+      <c r="F56">
+        <v>112</v>
+      </c>
+      <c r="G56">
+        <v>22</v>
+      </c>
+      <c r="H56">
+        <v>38</v>
+      </c>
+      <c r="I56">
+        <v>8</v>
+      </c>
+      <c r="J56" t="s">
+        <v>2175</v>
+      </c>
+      <c r="K56" t="s">
+        <v>2176</v>
+      </c>
+      <c r="L56" t="s">
+        <v>2177</v>
+      </c>
+    </row>
+    <row r="57" spans="4:12" x14ac:dyDescent="0.3">
+      <c r="D57" t="s">
+        <v>72</v>
+      </c>
+      <c r="E57" t="s">
+        <v>2178</v>
+      </c>
+      <c r="F57">
+        <v>135</v>
+      </c>
+      <c r="G57">
+        <v>22</v>
+      </c>
+      <c r="H57">
+        <v>16</v>
+      </c>
+      <c r="I57">
+        <v>24</v>
+      </c>
+      <c r="J57" t="s">
+        <v>2179</v>
+      </c>
+      <c r="K57" t="s">
+        <v>2180</v>
+      </c>
+      <c r="L57" t="s">
+        <v>2181</v>
+      </c>
+    </row>
+    <row r="58" spans="4:12" x14ac:dyDescent="0.3">
+      <c r="D58" t="s">
+        <v>72</v>
+      </c>
+      <c r="E58" t="s">
+        <v>2182</v>
+      </c>
+      <c r="F58">
+        <v>145</v>
+      </c>
+      <c r="G58">
+        <v>18</v>
+      </c>
+      <c r="H58">
+        <v>13</v>
+      </c>
+      <c r="I58">
+        <v>22</v>
+      </c>
+      <c r="J58" t="s">
+        <v>2183</v>
+      </c>
+      <c r="K58" t="s">
+        <v>2184</v>
+      </c>
+      <c r="L58" t="s">
+        <v>2185</v>
+      </c>
+    </row>
+    <row r="59" spans="4:12" x14ac:dyDescent="0.3">
+      <c r="D59" t="s">
+        <v>72</v>
+      </c>
+      <c r="E59" t="s">
+        <v>2186</v>
+      </c>
+      <c r="F59">
+        <v>125</v>
+      </c>
+      <c r="G59">
+        <v>24</v>
+      </c>
+      <c r="H59">
+        <v>18</v>
+      </c>
+      <c r="I59">
+        <v>22</v>
+      </c>
+      <c r="J59" t="s">
+        <v>2187</v>
+      </c>
+      <c r="K59" t="s">
+        <v>2188</v>
+      </c>
+      <c r="L59" t="s">
+        <v>2189</v>
+      </c>
+    </row>
+    <row r="60" spans="4:12" x14ac:dyDescent="0.3">
+      <c r="D60" t="s">
+        <v>72</v>
+      </c>
+      <c r="E60" t="s">
+        <v>2190</v>
+      </c>
+      <c r="F60">
+        <v>128</v>
+      </c>
+      <c r="G60">
+        <v>20</v>
+      </c>
+      <c r="H60">
+        <v>15</v>
+      </c>
+      <c r="I60">
+        <v>24</v>
+      </c>
+      <c r="J60" t="s">
+        <v>2191</v>
+      </c>
+      <c r="K60" t="s">
+        <v>2192</v>
+      </c>
+      <c r="L60" t="s">
+        <v>2193</v>
+      </c>
+    </row>
+    <row r="61" spans="4:12" x14ac:dyDescent="0.3">
+      <c r="D61" t="s">
+        <v>72</v>
+      </c>
+      <c r="E61" t="s">
+        <v>2194</v>
+      </c>
+      <c r="F61">
+        <v>140</v>
+      </c>
+      <c r="G61">
+        <v>21</v>
+      </c>
+      <c r="H61">
+        <v>15</v>
+      </c>
+      <c r="I61">
+        <v>26</v>
+      </c>
+      <c r="J61" t="s">
+        <v>2195</v>
+      </c>
+      <c r="K61" t="s">
+        <v>2196</v>
+      </c>
+      <c r="L61" t="s">
+        <v>2197</v>
+      </c>
+    </row>
+    <row r="62" spans="4:12" x14ac:dyDescent="0.3">
+      <c r="D62" t="s">
+        <v>72</v>
+      </c>
+      <c r="E62" t="s">
+        <v>2198</v>
+      </c>
+      <c r="F62">
+        <v>118</v>
+      </c>
+      <c r="G62">
+        <v>26</v>
+      </c>
+      <c r="H62">
+        <v>22</v>
+      </c>
+      <c r="I62">
+        <v>18</v>
+      </c>
+      <c r="J62" t="s">
+        <v>2199</v>
+      </c>
+      <c r="K62" t="s">
+        <v>2200</v>
+      </c>
+      <c r="L62" t="s">
+        <v>2201</v>
+      </c>
+    </row>
+    <row r="63" spans="4:12" x14ac:dyDescent="0.3">
+      <c r="D63" t="s">
+        <v>68</v>
+      </c>
+      <c r="E63" t="s">
+        <v>2202</v>
+      </c>
+      <c r="F63">
+        <v>118</v>
+      </c>
+      <c r="G63">
+        <v>34</v>
+      </c>
+      <c r="H63">
+        <v>22</v>
+      </c>
+      <c r="I63">
+        <v>14</v>
+      </c>
+      <c r="J63" t="s">
+        <v>2203</v>
+      </c>
+      <c r="K63" t="s">
+        <v>2204</v>
+      </c>
+      <c r="L63" t="s">
+        <v>2205</v>
+      </c>
+    </row>
+    <row r="64" spans="4:12" x14ac:dyDescent="0.3">
+      <c r="D64" t="s">
+        <v>68</v>
+      </c>
+      <c r="E64" t="s">
+        <v>2206</v>
+      </c>
+      <c r="F64">
+        <v>112</v>
+      </c>
+      <c r="G64">
+        <v>36</v>
+      </c>
+      <c r="H64">
+        <v>24</v>
+      </c>
+      <c r="I64">
+        <v>12</v>
+      </c>
+      <c r="J64" t="s">
+        <v>2207</v>
+      </c>
+      <c r="K64" t="s">
+        <v>2208</v>
+      </c>
+      <c r="L64" t="s">
+        <v>2209</v>
+      </c>
+    </row>
+    <row r="65" spans="4:12" x14ac:dyDescent="0.3">
+      <c r="D65" t="s">
+        <v>68</v>
+      </c>
+      <c r="E65" t="s">
+        <v>2210</v>
+      </c>
+      <c r="F65">
+        <v>125</v>
+      </c>
+      <c r="G65">
+        <v>30</v>
+      </c>
+      <c r="H65">
+        <v>20</v>
+      </c>
+      <c r="I65">
+        <v>16</v>
+      </c>
+      <c r="J65" t="s">
+        <v>2211</v>
+      </c>
+      <c r="K65" t="s">
+        <v>2212</v>
+      </c>
+      <c r="L65" t="s">
+        <v>2213</v>
+      </c>
+    </row>
+    <row r="66" spans="4:12" x14ac:dyDescent="0.3">
+      <c r="D66" t="s">
+        <v>68</v>
+      </c>
+      <c r="E66" t="s">
+        <v>2214</v>
+      </c>
+      <c r="F66">
+        <v>108</v>
+      </c>
+      <c r="G66">
+        <v>35</v>
+      </c>
+      <c r="H66">
+        <v>26</v>
+      </c>
+      <c r="I66">
+        <v>10</v>
+      </c>
+      <c r="J66" t="s">
+        <v>2215</v>
+      </c>
+      <c r="K66" t="s">
+        <v>2216</v>
+      </c>
+      <c r="L66" t="s">
+        <v>2217</v>
+      </c>
+    </row>
+    <row r="67" spans="4:12" x14ac:dyDescent="0.3">
+      <c r="D67" t="s">
+        <v>68</v>
+      </c>
+      <c r="E67" t="s">
+        <v>2218</v>
+      </c>
+      <c r="F67">
+        <v>115</v>
+      </c>
+      <c r="G67">
+        <v>32</v>
+      </c>
+      <c r="H67">
+        <v>25</v>
+      </c>
+      <c r="I67">
+        <v>12</v>
+      </c>
+      <c r="J67" t="s">
+        <v>2219</v>
+      </c>
+      <c r="K67" t="s">
+        <v>2220</v>
+      </c>
+      <c r="L67" t="s">
+        <v>2221</v>
+      </c>
+    </row>
+    <row r="68" spans="4:12" x14ac:dyDescent="0.3">
+      <c r="D68" t="s">
+        <v>68</v>
+      </c>
+      <c r="E68" t="s">
+        <v>2222</v>
+      </c>
+      <c r="F68">
+        <v>120</v>
+      </c>
+      <c r="G68">
+        <v>33</v>
+      </c>
+      <c r="H68">
+        <v>18</v>
+      </c>
+      <c r="I68">
+        <v>15</v>
+      </c>
+      <c r="J68" t="s">
+        <v>2223</v>
+      </c>
+      <c r="K68" t="s">
+        <v>2224</v>
+      </c>
+      <c r="L68" t="s">
+        <v>2225</v>
       </c>
     </row>
   </sheetData>
@@ -19660,12 +21369,6 @@
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="B29:B31"/>
-    <mergeCell ref="B14:B16"/>
-    <mergeCell ref="A8:A10"/>
-    <mergeCell ref="A26:A28"/>
-    <mergeCell ref="A17:A19"/>
-    <mergeCell ref="A20:A22"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A5:A7"/>
     <mergeCell ref="A23:A25"/>
@@ -19682,6 +21385,12 @@
     <mergeCell ref="B17:B19"/>
     <mergeCell ref="B23:B25"/>
     <mergeCell ref="A29:A31"/>
+    <mergeCell ref="B29:B31"/>
+    <mergeCell ref="B14:B16"/>
+    <mergeCell ref="A8:A10"/>
+    <mergeCell ref="A26:A28"/>
+    <mergeCell ref="A17:A19"/>
+    <mergeCell ref="A20:A22"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <ignoredErrors>
@@ -21274,7 +22983,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
@@ -21722,6 +23431,29 @@
       </c>
       <c r="G22" t="s">
         <v>760</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>701</v>
+      </c>
+      <c r="B23" t="s">
+        <v>2312</v>
+      </c>
+      <c r="C23" t="s">
+        <v>2258</v>
+      </c>
+      <c r="D23" t="s">
+        <v>2313</v>
+      </c>
+      <c r="E23" t="s">
+        <v>2314</v>
+      </c>
+      <c r="F23" t="s">
+        <v>2315</v>
+      </c>
+      <c r="G23" t="s">
+        <v>2316</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix dodge-credit gaps for stackable passives, add REGENERATION enemy skill, redesign Party stat radar chart
- Extend the artifact/weapon dodge -> form-bonus credit hook (previously only
  covering a few forms) to also cover PANDA-NINJA, BUNNY-GHOST, CAT-GHOST on
  the player side, their Fusion Echo variants, and add the equivalent hook for
  the enemy mirror side (fk2) which had none at all.
- Add new Enemy Skill "REGENERATION" (regen_cleanse): heals 3% MaxHP and
  cleanses one of its own debuffs every turn. Logged in SYMBEAST_Evolve_Forms.xlsx.
- Redesign the Party screen's pet stat display as a diamond/radar chart
  (HP/ATK/SPD/DEF) next to the sprite, with sqrt-scaled axes so the shape
  reflects real stat differences between pets instead of every trained pet
  looking maxed out, plus nav arrows overlaid on the sprite so the chart's
  size doesn't shrink the character.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SYMBEAST_Evolve_Forms.xlsx
+++ b/SYMBEAST_Evolve_Forms.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\skyit\Desktop\Symbeast-main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34B510CA-2E55-47F7-A5AD-9F249BF4CEA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCF1E4BF-3AA6-4C0B-9E7D-3BA55DF767B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="11" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3862" uniqueCount="2317">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3869" uniqueCount="2322">
   <si>
     <t>SYMBEAST — Evolved Forms (Stage 1, 10 forms)</t>
   </si>
@@ -6987,6 +6987,21 @@
   </si>
   <si>
     <t>20% โอกาสทำให้ผู้เล่นตาบอดเมื่อโจมตีโดน (โจมตีพลาด 50% นาน 3 เทิร์น)</t>
+  </si>
+  <si>
+    <t>regen_cleanse</t>
+  </si>
+  <si>
+    <t>REGENERATION</t>
+  </si>
+  <si>
+    <t>ฟื้นฟู</t>
+  </si>
+  <si>
+    <t>Heals 3% MaxHP and cleanses its own debuffs every turn</t>
+  </si>
+  <si>
+    <t>ฟื้นฟู HP 3% และล้างดีบัพของตัวเองทุกเทิร์น</t>
   </si>
 </sst>
 </file>
@@ -21369,6 +21384,12 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="B29:B31"/>
+    <mergeCell ref="B14:B16"/>
+    <mergeCell ref="A8:A10"/>
+    <mergeCell ref="A26:A28"/>
+    <mergeCell ref="A17:A19"/>
+    <mergeCell ref="A20:A22"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A5:A7"/>
     <mergeCell ref="A23:A25"/>
@@ -21385,12 +21406,6 @@
     <mergeCell ref="B17:B19"/>
     <mergeCell ref="B23:B25"/>
     <mergeCell ref="A29:A31"/>
-    <mergeCell ref="B29:B31"/>
-    <mergeCell ref="B14:B16"/>
-    <mergeCell ref="A8:A10"/>
-    <mergeCell ref="A26:A28"/>
-    <mergeCell ref="A17:A19"/>
-    <mergeCell ref="A20:A22"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <ignoredErrors>
@@ -22983,7 +22998,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
@@ -23454,6 +23469,29 @@
       </c>
       <c r="G23" t="s">
         <v>2316</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>717</v>
+      </c>
+      <c r="B24" t="s">
+        <v>2317</v>
+      </c>
+      <c r="C24" t="s">
+        <v>486</v>
+      </c>
+      <c r="D24" t="s">
+        <v>2318</v>
+      </c>
+      <c r="E24" t="s">
+        <v>2319</v>
+      </c>
+      <c r="F24" t="s">
+        <v>2320</v>
+      </c>
+      <c r="G24" t="s">
+        <v>2321</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Expand Fire/Poison/Freeze Absorb systems + rework CHILL-SHIELDWING & GAIA-SHIELDWING skills
- Fire Absorb: add IFRIT-GHOST, DRAGON-TAMER-GHOST, BAHAMUT-GHOST, DRAGON-KNIGHT-GHOST, TRICKFOX-GHOST

- Freeze Absorb: SHIVA-GHOST, CRYSTAWOLF-BASTION, PENGUIN-GHOST, CHILL-SHIELDWING, GAIA-SHIELDWING

- Poison Absorb: 9 monsters (SLIME, FORTRESS variants, GREEN-SENTINEL, ARC-DEMON, LEAPFROG, GRAVE-SPECTER)

- Rework CHILL-SHIELDWING: 3T dodge 100%, pierce DEF ATK+50%, 50% freeze; OD freeze every turn

- Rework GAIA-SHIELDWING: 10% freeze on hit, 3T heal 15% MaxHP + ATK/DEF+20%

- Fix scope bugs: GAIA OD/branch eFreezeAbsorb before declaration; SHIVA OD missing CHILL/GAIA

- Update Excel (TH/EN) for CHILL/GAIA skill descriptions
</commit_message>
<xml_diff>
--- a/SYMBEAST_Evolve_Forms.xlsx
+++ b/SYMBEAST_Evolve_Forms.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="600" firstSheet="11" activeTab="15" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="600" firstSheet="1" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Evolved Forms" sheetId="1" state="visible" r:id="rId1"/>
@@ -13718,12 +13718,12 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Every 3 turns: dodges 50% and attacks through DEF with ATK +25%</t>
+          <t>Every 3 turns: dodges 50%, attacks through DEF with ATK +25%, 25% chance to freeze the enemy</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>ทุก 3 เทิร์น: หลบ 50% และโจมตีทะลุ DEF ด้วย ATK+25%</t>
+          <t>ทุก 3 เทิร์น: หลบ 50% โจมตีทะลุ DEF ด้วย ATK+25% และโอกาส 25% แช่แข็งศัตรู</t>
         </is>
       </c>
     </row>
@@ -13745,12 +13745,12 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Every 3 rounds: recovers 8% of Max HP and ATK/DEF +10% that round</t>
+          <t>Every 3 rounds: recovers 8% of Max HP and ATK/DEF +10% that round; 5% chance to freeze the enemy on hit</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>ทุก 3 รอบ: ฟื้น HP 8% ของ Max HP และ ATK/DEF+10% ในรอบนั้น</t>
+          <t>ทุก 3 รอบ: ฟื้น HP 8% ของ Max HP และ ATK/DEF+10% ในรอบนั้น; 5% โอกาสแช่แข็งศัตรูเมื่อโจมตี</t>
         </is>
       </c>
     </row>
@@ -18700,7 +18700,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>ทุก 3 เทิร์น จะหลบการโจมตีได้ 100% และโจมตีทะลุ DEF ด้วย ATK+50%</t>
+          <t>ทุก 3 เทิร์น จะหลบการโจมตีได้ 100% และโจมตีทะลุ DEF ด้วย ATK+50% และมีโอกาส 50% แช่แข็งศัตรู</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -18710,7 +18710,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>โจมตี ×3.0 ทะลุ DEF + หลบการโจมตีสมบูรณ์เทิร์นนี้ จากนั้น 3 เทิร์น: โอกาสหลบ +30%, โจมตีทะลุ DEF ต่อเนื่อง</t>
+          <t>โจมตี ×3.0 ทะลุ DEF + หลบการโจมตีเทิร์นนี้ จากนั้น 3 เทิร์น: โอกาสหลบ +30%, โจมตีทะลุ DEF, 50% แช่แข็งศัตรู</t>
         </is>
       </c>
     </row>
@@ -18739,7 +18739,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>ทุก 3 รอบ: ฟื้น HP 15% ของ Max HP และ ATK/DEF+20% ในรอบนั้น</t>
+          <t>มีโอกาส 10% แช่แข็งศัตรู และทุก 3 รอบ: ฟื้น HP 15% ของ Max HP และ ATK/DEF+20% ในรอบนั้น</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -18749,7 +18749,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>โจมตี ×3.0 ทะลุ DEF + ฟื้นฟู HP 20% เทิร์นนี้ จากนั้น ATK/DEF +30% และฟื้นฟู HP 10% ต่อเทิร์น นาน 3 เทิร์น</t>
+          <t>โจมตี ×3.0 ทะลุ DEF + ฟื้นฟู HP 20% เทิร์นนี้ จากนั้น ATK/DEF +30%, ฟื้นฟู HP 10% ต่อเทิร์น, 10% แช่แข็งศัตรู นาน 3 เทิร์น</t>
         </is>
       </c>
     </row>
@@ -21138,7 +21138,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>โจมตี ×3.0 ทะลุ DEF + หลบการโจมตีสมบูรณ์เทิร์นนี้ → จากนั้น 3 เทิร์น: โอกาสหลบ +30%, โจมตีทะลุ DEF ต่อเนื่อง</t>
+          <t>โจมตี ×3.0 ทะลุ DEF + หลบการโจมตีเทิร์นนี้ → จากนั้น 3 เทิร์น: โอกาสหลบ +30%, โจมตีทะลุ DEF, 50% แช่แข็งศัตรู</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Revert "Expand Fire/Poison/Freeze Absorb systems + rework CHILL-SHIELDWING & GAIA-SHIELDWING skills"
This reverts commit 4d4a8c71e2016e14b24aebb9a8b361e2e5f2c7af.
</commit_message>
<xml_diff>
--- a/SYMBEAST_Evolve_Forms.xlsx
+++ b/SYMBEAST_Evolve_Forms.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="600" firstSheet="1" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="600" firstSheet="11" activeTab="15" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Evolved Forms" sheetId="1" state="visible" r:id="rId1"/>
@@ -13718,12 +13718,12 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Every 3 turns: dodges 50%, attacks through DEF with ATK +25%, 25% chance to freeze the enemy</t>
+          <t>Every 3 turns: dodges 50% and attacks through DEF with ATK +25%</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>ทุก 3 เทิร์น: หลบ 50% โจมตีทะลุ DEF ด้วย ATK+25% และโอกาส 25% แช่แข็งศัตรู</t>
+          <t>ทุก 3 เทิร์น: หลบ 50% และโจมตีทะลุ DEF ด้วย ATK+25%</t>
         </is>
       </c>
     </row>
@@ -13745,12 +13745,12 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Every 3 rounds: recovers 8% of Max HP and ATK/DEF +10% that round; 5% chance to freeze the enemy on hit</t>
+          <t>Every 3 rounds: recovers 8% of Max HP and ATK/DEF +10% that round</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>ทุก 3 รอบ: ฟื้น HP 8% ของ Max HP และ ATK/DEF+10% ในรอบนั้น; 5% โอกาสแช่แข็งศัตรูเมื่อโจมตี</t>
+          <t>ทุก 3 รอบ: ฟื้น HP 8% ของ Max HP และ ATK/DEF+10% ในรอบนั้น</t>
         </is>
       </c>
     </row>
@@ -18700,7 +18700,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>ทุก 3 เทิร์น จะหลบการโจมตีได้ 100% และโจมตีทะลุ DEF ด้วย ATK+50% และมีโอกาส 50% แช่แข็งศัตรู</t>
+          <t>ทุก 3 เทิร์น จะหลบการโจมตีได้ 100% และโจมตีทะลุ DEF ด้วย ATK+50%</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -18710,7 +18710,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>โจมตี ×3.0 ทะลุ DEF + หลบการโจมตีเทิร์นนี้ จากนั้น 3 เทิร์น: โอกาสหลบ +30%, โจมตีทะลุ DEF, 50% แช่แข็งศัตรู</t>
+          <t>โจมตี ×3.0 ทะลุ DEF + หลบการโจมตีสมบูรณ์เทิร์นนี้ จากนั้น 3 เทิร์น: โอกาสหลบ +30%, โจมตีทะลุ DEF ต่อเนื่อง</t>
         </is>
       </c>
     </row>
@@ -18739,7 +18739,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>มีโอกาส 10% แช่แข็งศัตรู และทุก 3 รอบ: ฟื้น HP 15% ของ Max HP และ ATK/DEF+20% ในรอบนั้น</t>
+          <t>ทุก 3 รอบ: ฟื้น HP 15% ของ Max HP และ ATK/DEF+20% ในรอบนั้น</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -18749,7 +18749,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>โจมตี ×3.0 ทะลุ DEF + ฟื้นฟู HP 20% เทิร์นนี้ จากนั้น ATK/DEF +30%, ฟื้นฟู HP 10% ต่อเทิร์น, 10% แช่แข็งศัตรู นาน 3 เทิร์น</t>
+          <t>โจมตี ×3.0 ทะลุ DEF + ฟื้นฟู HP 20% เทิร์นนี้ จากนั้น ATK/DEF +30% และฟื้นฟู HP 10% ต่อเทิร์น นาน 3 เทิร์น</t>
         </is>
       </c>
     </row>
@@ -21138,7 +21138,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>โจมตี ×3.0 ทะลุ DEF + หลบการโจมตีเทิร์นนี้ → จากนั้น 3 เทิร์น: โอกาสหลบ +30%, โจมตีทะลุ DEF, 50% แช่แข็งศัตรู</t>
+          <t>โจมตี ×3.0 ทะลุ DEF + หลบการโจมตีสมบูรณ์เทิร์นนี้ → จากนั้น 3 เทิร์น: โอกาสหลบ +30%, โจมตีทะลุ DEF ต่อเนื่อง</t>
         </is>
       </c>
     </row>

</xml_diff>